<commit_message>
Add focused sector stock sheet
</commit_message>
<xml_diff>
--- a/INDmoney-All-Sectors-Under-20-Review.xlsx
+++ b/INDmoney-All-Sectors-Under-20-Review.xlsx
@@ -5,13 +5,14 @@
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
     <sheet sheetId="1" name="Stocks under 20Rs" state="visible" r:id="rId4"/>
+    <sheet sheetId="2" name="Focus Sectors" state="visible" r:id="rId5"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1393" uniqueCount="987">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1974" uniqueCount="1000">
   <si>
     <t>Sector</t>
   </si>
@@ -2972,13 +2973,52 @@
   </si>
   <si>
     <t>https://www.indmoney.com/stocks/centrum-capital-ltd-share-price</t>
+  </si>
+  <si>
+    <t>Focus Group</t>
+  </si>
+  <si>
+    <t>Metal Type</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>Metals</t>
+  </si>
+  <si>
+    <t>Steel / Other</t>
+  </si>
+  <si>
+    <t>Watchlist - Infrastructure</t>
+  </si>
+  <si>
+    <t>Brass</t>
+  </si>
+  <si>
+    <t>FMCG</t>
+  </si>
+  <si>
+    <t>Steel / Ferro-alloys</t>
+  </si>
+  <si>
+    <t>Copper</t>
+  </si>
+  <si>
+    <t>Aluminium</t>
+  </si>
+  <si>
+    <t>Watchlist - Defence</t>
+  </si>
+  <si>
+    <t>Metal types follow INDmoney company descriptions. No company explicitly focused on zinc and no Railway-category stock appeared below ₹20 in the 47 source sectors. Additional watchlist groups are not investment recommendations.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -2993,6 +3033,10 @@
     <font>
       <u/>
       <color rgb="FF0000FF"/>
+    </font>
+    <font>
+      <i/>
+      <color rgb="FF666666"/>
     </font>
   </fonts>
   <fills count="3">
@@ -3020,7 +3064,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -3028,6 +3072,9 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -17687,4 +17734,4280 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:O115"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="40" customWidth="1"/>
+    <col min="2" max="2" width="20" customWidth="1"/>
+    <col min="3" max="3" width="40" customWidth="1"/>
+    <col min="4" max="4" width="38" customWidth="1"/>
+    <col min="5" max="5" width="12" customWidth="1"/>
+    <col min="6" max="6" width="18" customWidth="1"/>
+    <col min="7" max="7" width="14" customWidth="1"/>
+    <col min="8" max="11" width="12" customWidth="1"/>
+    <col min="12" max="14" width="14" customWidth="1"/>
+    <col min="15" max="15" width="58" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="32" customHeight="1" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>987</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>988</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B2" t="s">
+        <v>989</v>
+      </c>
+      <c r="C2" t="s">
+        <v>24</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="E2" s="3">
+        <v>0.22</v>
+      </c>
+      <c r="F2" s="4">
+        <v>25.95</v>
+      </c>
+      <c r="G2" s="3"/>
+      <c r="H2" s="3"/>
+      <c r="I2" s="3">
+        <v>2.42</v>
+      </c>
+      <c r="J2" s="3">
+        <v>3.81</v>
+      </c>
+      <c r="K2" s="3"/>
+      <c r="L2" s="3"/>
+      <c r="M2" s="3"/>
+      <c r="N2" s="3"/>
+      <c r="O2" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>24</v>
+      </c>
+      <c r="B3" t="s">
+        <v>989</v>
+      </c>
+      <c r="C3" t="s">
+        <v>24</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="E3" s="3">
+        <v>0.27</v>
+      </c>
+      <c r="F3" s="4">
+        <v>22.93</v>
+      </c>
+      <c r="G3" s="3"/>
+      <c r="H3" s="3"/>
+      <c r="I3" s="3">
+        <v>1.76</v>
+      </c>
+      <c r="J3" s="3">
+        <v>3.55</v>
+      </c>
+      <c r="K3" s="3"/>
+      <c r="L3" s="3"/>
+      <c r="M3" s="3"/>
+      <c r="N3" s="3"/>
+      <c r="O3" s="2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>24</v>
+      </c>
+      <c r="B4" t="s">
+        <v>989</v>
+      </c>
+      <c r="C4" t="s">
+        <v>24</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="E4" s="3">
+        <v>0.37</v>
+      </c>
+      <c r="F4" s="4">
+        <v>36.55</v>
+      </c>
+      <c r="G4" s="3"/>
+      <c r="H4" s="3"/>
+      <c r="I4" s="3">
+        <v>0</v>
+      </c>
+      <c r="J4" s="3">
+        <v>0</v>
+      </c>
+      <c r="K4" s="3"/>
+      <c r="L4" s="3"/>
+      <c r="M4" s="3"/>
+      <c r="N4" s="3"/>
+      <c r="O4" s="2" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>990</v>
+      </c>
+      <c r="B5" t="s">
+        <v>991</v>
+      </c>
+      <c r="C5" t="s">
+        <v>46</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="E5" s="3">
+        <v>0.6</v>
+      </c>
+      <c r="F5" s="4">
+        <v>0.37</v>
+      </c>
+      <c r="G5" s="3"/>
+      <c r="H5" s="3"/>
+      <c r="I5" s="3">
+        <v>0</v>
+      </c>
+      <c r="J5" s="3">
+        <v>0</v>
+      </c>
+      <c r="K5" s="3"/>
+      <c r="L5" s="3"/>
+      <c r="M5" s="3"/>
+      <c r="N5" s="3"/>
+      <c r="O5" s="2" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>990</v>
+      </c>
+      <c r="B6" t="s">
+        <v>991</v>
+      </c>
+      <c r="C6" t="s">
+        <v>46</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="E6" s="3">
+        <v>0.82</v>
+      </c>
+      <c r="F6" s="4">
+        <v>24.29</v>
+      </c>
+      <c r="G6" s="3"/>
+      <c r="H6" s="3"/>
+      <c r="I6" s="3">
+        <v>6.08</v>
+      </c>
+      <c r="J6" s="3">
+        <v>4.64</v>
+      </c>
+      <c r="K6" s="3"/>
+      <c r="L6" s="3"/>
+      <c r="M6" s="3"/>
+      <c r="N6" s="3"/>
+      <c r="O6" s="2" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>992</v>
+      </c>
+      <c r="B7" t="s">
+        <v>989</v>
+      </c>
+      <c r="C7" t="s">
+        <v>51</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="E7" s="3">
+        <v>0.85</v>
+      </c>
+      <c r="F7" s="4">
+        <v>95.38</v>
+      </c>
+      <c r="G7" s="3"/>
+      <c r="H7" s="3"/>
+      <c r="I7" s="3">
+        <v>3.49</v>
+      </c>
+      <c r="J7" s="3">
+        <v>2.41</v>
+      </c>
+      <c r="K7" s="3"/>
+      <c r="L7" s="3"/>
+      <c r="M7" s="3"/>
+      <c r="N7" s="3"/>
+      <c r="O7" s="2" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>990</v>
+      </c>
+      <c r="B8" t="s">
+        <v>993</v>
+      </c>
+      <c r="C8" t="s">
+        <v>72</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="E8" s="3">
+        <v>1.2</v>
+      </c>
+      <c r="F8" s="4">
+        <v>25.36</v>
+      </c>
+      <c r="G8" s="3"/>
+      <c r="H8" s="3"/>
+      <c r="I8" s="3">
+        <v>4.34</v>
+      </c>
+      <c r="J8" s="3">
+        <v>1.27</v>
+      </c>
+      <c r="K8" s="3"/>
+      <c r="L8" s="3"/>
+      <c r="M8" s="3"/>
+      <c r="N8" s="3"/>
+      <c r="O8" s="2" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>992</v>
+      </c>
+      <c r="B9" t="s">
+        <v>989</v>
+      </c>
+      <c r="C9" t="s">
+        <v>51</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="E9" s="3">
+        <v>1.3</v>
+      </c>
+      <c r="F9" s="4">
+        <v>74.73</v>
+      </c>
+      <c r="G9" s="3"/>
+      <c r="H9" s="3"/>
+      <c r="I9" s="3">
+        <v>5.03</v>
+      </c>
+      <c r="J9" s="3">
+        <v>1.96</v>
+      </c>
+      <c r="K9" s="3"/>
+      <c r="L9" s="3"/>
+      <c r="M9" s="3"/>
+      <c r="N9" s="3"/>
+      <c r="O9" s="2" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>104</v>
+      </c>
+      <c r="B10" t="s">
+        <v>989</v>
+      </c>
+      <c r="C10" t="s">
+        <v>104</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="E10" s="3">
+        <v>1.74</v>
+      </c>
+      <c r="F10" s="4">
+        <v>9.51</v>
+      </c>
+      <c r="G10" s="3"/>
+      <c r="H10" s="3"/>
+      <c r="I10" s="3">
+        <v>0</v>
+      </c>
+      <c r="J10" s="3">
+        <v>0</v>
+      </c>
+      <c r="K10" s="3"/>
+      <c r="L10" s="3"/>
+      <c r="M10" s="3"/>
+      <c r="N10" s="3"/>
+      <c r="O10" s="2" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>992</v>
+      </c>
+      <c r="B11" t="s">
+        <v>989</v>
+      </c>
+      <c r="C11" t="s">
+        <v>51</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="E11" s="3">
+        <v>1.87</v>
+      </c>
+      <c r="F11" s="4">
+        <v>61.52</v>
+      </c>
+      <c r="G11" s="3"/>
+      <c r="H11" s="3"/>
+      <c r="I11" s="3">
+        <v>0</v>
+      </c>
+      <c r="J11" s="3">
+        <v>0</v>
+      </c>
+      <c r="K11" s="3"/>
+      <c r="L11" s="3"/>
+      <c r="M11" s="3"/>
+      <c r="N11" s="3"/>
+      <c r="O11" s="2" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>990</v>
+      </c>
+      <c r="B12" t="s">
+        <v>991</v>
+      </c>
+      <c r="C12" t="s">
+        <v>46</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="E12" s="3">
+        <v>2.06</v>
+      </c>
+      <c r="F12" s="4">
+        <v>29.07</v>
+      </c>
+      <c r="G12" s="3"/>
+      <c r="H12" s="3"/>
+      <c r="I12" s="3">
+        <v>0</v>
+      </c>
+      <c r="J12" s="3">
+        <v>0</v>
+      </c>
+      <c r="K12" s="3"/>
+      <c r="L12" s="3"/>
+      <c r="M12" s="3"/>
+      <c r="N12" s="3"/>
+      <c r="O12" s="2" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>992</v>
+      </c>
+      <c r="B13" t="s">
+        <v>989</v>
+      </c>
+      <c r="C13" t="s">
+        <v>51</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="E13" s="3">
+        <v>2.13</v>
+      </c>
+      <c r="F13" s="4">
+        <v>92.69</v>
+      </c>
+      <c r="G13" s="3"/>
+      <c r="H13" s="3"/>
+      <c r="I13" s="3">
+        <v>0</v>
+      </c>
+      <c r="J13" s="3">
+        <v>0</v>
+      </c>
+      <c r="K13" s="3"/>
+      <c r="L13" s="3"/>
+      <c r="M13" s="3"/>
+      <c r="N13" s="3"/>
+      <c r="O13" s="2" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>994</v>
+      </c>
+      <c r="B14" t="s">
+        <v>989</v>
+      </c>
+      <c r="C14" t="s">
+        <v>146</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="E14" s="3">
+        <v>2.26</v>
+      </c>
+      <c r="F14" s="4">
+        <v>383.27</v>
+      </c>
+      <c r="G14" s="3"/>
+      <c r="H14" s="3"/>
+      <c r="I14" s="3">
+        <v>6.28</v>
+      </c>
+      <c r="J14" s="3">
+        <v>3.12</v>
+      </c>
+      <c r="K14" s="3"/>
+      <c r="L14" s="3"/>
+      <c r="M14" s="3"/>
+      <c r="N14" s="3"/>
+      <c r="O14" s="2" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>104</v>
+      </c>
+      <c r="B15" t="s">
+        <v>989</v>
+      </c>
+      <c r="C15" t="s">
+        <v>104</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="E15" s="3">
+        <v>2.34</v>
+      </c>
+      <c r="F15" s="4">
+        <v>18.18</v>
+      </c>
+      <c r="G15" s="3"/>
+      <c r="H15" s="3"/>
+      <c r="I15" s="3">
+        <v>0</v>
+      </c>
+      <c r="J15" s="3">
+        <v>0</v>
+      </c>
+      <c r="K15" s="3"/>
+      <c r="L15" s="3"/>
+      <c r="M15" s="3"/>
+      <c r="N15" s="3"/>
+      <c r="O15" s="2" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>992</v>
+      </c>
+      <c r="B16" t="s">
+        <v>989</v>
+      </c>
+      <c r="C16" t="s">
+        <v>158</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="E16" s="3">
+        <v>2.51</v>
+      </c>
+      <c r="F16" s="4">
+        <v>396.38</v>
+      </c>
+      <c r="G16" s="3"/>
+      <c r="H16" s="3"/>
+      <c r="I16" s="3">
+        <v>0</v>
+      </c>
+      <c r="J16" s="3">
+        <v>0</v>
+      </c>
+      <c r="K16" s="3"/>
+      <c r="L16" s="3"/>
+      <c r="M16" s="3"/>
+      <c r="N16" s="3"/>
+      <c r="O16" s="2" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="17" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>992</v>
+      </c>
+      <c r="B17" t="s">
+        <v>989</v>
+      </c>
+      <c r="C17" t="s">
+        <v>51</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>169</v>
+      </c>
+      <c r="E17" s="3">
+        <v>2.62</v>
+      </c>
+      <c r="F17" s="4">
+        <v>92.28</v>
+      </c>
+      <c r="G17" s="3"/>
+      <c r="H17" s="3"/>
+      <c r="I17" s="3">
+        <v>-1.52</v>
+      </c>
+      <c r="J17" s="3">
+        <v>-9.2</v>
+      </c>
+      <c r="K17" s="3"/>
+      <c r="L17" s="3"/>
+      <c r="M17" s="3"/>
+      <c r="N17" s="3"/>
+      <c r="O17" s="2" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="18" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>990</v>
+      </c>
+      <c r="B18" t="s">
+        <v>991</v>
+      </c>
+      <c r="C18" t="s">
+        <v>190</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>191</v>
+      </c>
+      <c r="E18" s="3">
+        <v>3.03</v>
+      </c>
+      <c r="F18" s="4">
+        <v>119.67</v>
+      </c>
+      <c r="G18" s="3"/>
+      <c r="H18" s="3"/>
+      <c r="I18" s="3">
+        <v>0</v>
+      </c>
+      <c r="J18" s="3">
+        <v>0</v>
+      </c>
+      <c r="K18" s="3"/>
+      <c r="L18" s="3"/>
+      <c r="M18" s="3"/>
+      <c r="N18" s="3"/>
+      <c r="O18" s="2" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="19" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>990</v>
+      </c>
+      <c r="B19" t="s">
+        <v>991</v>
+      </c>
+      <c r="C19" t="s">
+        <v>190</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="E19" s="3">
+        <v>3.03</v>
+      </c>
+      <c r="F19" s="4">
+        <v>300.69</v>
+      </c>
+      <c r="G19" s="3"/>
+      <c r="H19" s="3"/>
+      <c r="I19" s="3">
+        <v>4.23</v>
+      </c>
+      <c r="J19" s="3">
+        <v>3.43</v>
+      </c>
+      <c r="K19" s="3"/>
+      <c r="L19" s="3"/>
+      <c r="M19" s="3"/>
+      <c r="N19" s="3"/>
+      <c r="O19" s="2" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="20" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>990</v>
+      </c>
+      <c r="B20" t="s">
+        <v>995</v>
+      </c>
+      <c r="C20" t="s">
+        <v>190</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>195</v>
+      </c>
+      <c r="E20" s="3">
+        <v>3.07</v>
+      </c>
+      <c r="F20" s="4">
+        <v>59.25</v>
+      </c>
+      <c r="G20" s="3"/>
+      <c r="H20" s="3"/>
+      <c r="I20" s="3">
+        <v>0</v>
+      </c>
+      <c r="J20" s="3">
+        <v>0</v>
+      </c>
+      <c r="K20" s="3"/>
+      <c r="L20" s="3"/>
+      <c r="M20" s="3"/>
+      <c r="N20" s="3"/>
+      <c r="O20" s="2" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="21" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>994</v>
+      </c>
+      <c r="B21" t="s">
+        <v>989</v>
+      </c>
+      <c r="C21" t="s">
+        <v>146</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="E21" s="3">
+        <v>3.08</v>
+      </c>
+      <c r="F21" s="4">
+        <v>330.83</v>
+      </c>
+      <c r="G21" s="3"/>
+      <c r="H21" s="3"/>
+      <c r="I21" s="3">
+        <v>3.71</v>
+      </c>
+      <c r="J21" s="3">
+        <v>2.36</v>
+      </c>
+      <c r="K21" s="3"/>
+      <c r="L21" s="3"/>
+      <c r="M21" s="3"/>
+      <c r="N21" s="3"/>
+      <c r="O21" s="2" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="22" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>990</v>
+      </c>
+      <c r="B22" t="s">
+        <v>996</v>
+      </c>
+      <c r="C22" t="s">
+        <v>199</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>200</v>
+      </c>
+      <c r="E22" s="3">
+        <v>3.08</v>
+      </c>
+      <c r="F22" s="4">
+        <v>85.16</v>
+      </c>
+      <c r="G22" s="3"/>
+      <c r="H22" s="3"/>
+      <c r="I22" s="3">
+        <v>4.85</v>
+      </c>
+      <c r="J22" s="3">
+        <v>-0.21</v>
+      </c>
+      <c r="K22" s="3"/>
+      <c r="L22" s="3"/>
+      <c r="M22" s="3"/>
+      <c r="N22" s="3"/>
+      <c r="O22" s="2" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="23" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>994</v>
+      </c>
+      <c r="B23" t="s">
+        <v>989</v>
+      </c>
+      <c r="C23" t="s">
+        <v>146</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>206</v>
+      </c>
+      <c r="E23" s="3">
+        <v>3.44</v>
+      </c>
+      <c r="F23" s="4">
+        <v>424.04</v>
+      </c>
+      <c r="G23" s="3"/>
+      <c r="H23" s="3"/>
+      <c r="I23" s="3">
+        <v>8.46</v>
+      </c>
+      <c r="J23" s="3">
+        <v>4.07</v>
+      </c>
+      <c r="K23" s="3"/>
+      <c r="L23" s="3"/>
+      <c r="M23" s="3"/>
+      <c r="N23" s="3"/>
+      <c r="O23" s="2" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="24" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>992</v>
+      </c>
+      <c r="B24" t="s">
+        <v>989</v>
+      </c>
+      <c r="C24" t="s">
+        <v>51</v>
+      </c>
+      <c r="D24" s="2" t="s">
+        <v>210</v>
+      </c>
+      <c r="E24" s="3">
+        <v>3.56</v>
+      </c>
+      <c r="F24" s="4">
+        <v>66.29</v>
+      </c>
+      <c r="G24" s="3"/>
+      <c r="H24" s="3"/>
+      <c r="I24" s="3">
+        <v>0</v>
+      </c>
+      <c r="J24" s="3">
+        <v>0</v>
+      </c>
+      <c r="K24" s="3"/>
+      <c r="L24" s="3"/>
+      <c r="M24" s="3"/>
+      <c r="N24" s="3"/>
+      <c r="O24" s="2" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="25" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>990</v>
+      </c>
+      <c r="B25" t="s">
+        <v>991</v>
+      </c>
+      <c r="C25" t="s">
+        <v>190</v>
+      </c>
+      <c r="D25" s="2" t="s">
+        <v>212</v>
+      </c>
+      <c r="E25" s="3">
+        <v>3.56</v>
+      </c>
+      <c r="F25" s="4">
+        <v>62.3</v>
+      </c>
+      <c r="G25" s="3"/>
+      <c r="H25" s="3"/>
+      <c r="I25" s="3">
+        <v>1.01</v>
+      </c>
+      <c r="J25" s="3">
+        <v>0.72</v>
+      </c>
+      <c r="K25" s="3"/>
+      <c r="L25" s="3"/>
+      <c r="M25" s="3"/>
+      <c r="N25" s="3"/>
+      <c r="O25" s="2" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="26" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>990</v>
+      </c>
+      <c r="B26" t="s">
+        <v>997</v>
+      </c>
+      <c r="C26" t="s">
+        <v>220</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>221</v>
+      </c>
+      <c r="E26" s="3">
+        <v>3.7</v>
+      </c>
+      <c r="F26" s="4">
+        <v>46</v>
+      </c>
+      <c r="G26" s="3"/>
+      <c r="H26" s="3"/>
+      <c r="I26" s="3">
+        <v>10.2</v>
+      </c>
+      <c r="J26" s="3">
+        <v>8.89</v>
+      </c>
+      <c r="K26" s="3"/>
+      <c r="L26" s="3"/>
+      <c r="M26" s="3"/>
+      <c r="N26" s="3"/>
+      <c r="O26" s="2" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="27" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>990</v>
+      </c>
+      <c r="B27" t="s">
+        <v>991</v>
+      </c>
+      <c r="C27" t="s">
+        <v>190</v>
+      </c>
+      <c r="D27" s="2" t="s">
+        <v>242</v>
+      </c>
+      <c r="E27" s="3">
+        <v>4.02</v>
+      </c>
+      <c r="F27" s="4">
+        <v>43.8</v>
+      </c>
+      <c r="G27" s="3"/>
+      <c r="H27" s="3"/>
+      <c r="I27" s="3">
+        <v>3.56</v>
+      </c>
+      <c r="J27" s="3">
+        <v>2.5</v>
+      </c>
+      <c r="K27" s="3"/>
+      <c r="L27" s="3"/>
+      <c r="M27" s="3"/>
+      <c r="N27" s="3"/>
+      <c r="O27" s="2" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="28" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>990</v>
+      </c>
+      <c r="B28" t="s">
+        <v>991</v>
+      </c>
+      <c r="C28" t="s">
+        <v>190</v>
+      </c>
+      <c r="D28" s="2" t="s">
+        <v>252</v>
+      </c>
+      <c r="E28" s="3">
+        <v>4.1</v>
+      </c>
+      <c r="F28" s="4">
+        <v>134.89</v>
+      </c>
+      <c r="G28" s="3"/>
+      <c r="H28" s="3"/>
+      <c r="I28" s="3">
+        <v>0</v>
+      </c>
+      <c r="J28" s="3">
+        <v>0</v>
+      </c>
+      <c r="K28" s="3"/>
+      <c r="L28" s="3"/>
+      <c r="M28" s="3"/>
+      <c r="N28" s="3"/>
+      <c r="O28" s="2" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="29" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>990</v>
+      </c>
+      <c r="B29" t="s">
+        <v>991</v>
+      </c>
+      <c r="C29" t="s">
+        <v>190</v>
+      </c>
+      <c r="D29" s="2" t="s">
+        <v>258</v>
+      </c>
+      <c r="E29" s="3">
+        <v>4.13</v>
+      </c>
+      <c r="F29" s="4">
+        <v>721.9</v>
+      </c>
+      <c r="G29" s="3"/>
+      <c r="H29" s="3"/>
+      <c r="I29" s="3">
+        <v>10.05</v>
+      </c>
+      <c r="J29" s="3">
+        <v>5.83</v>
+      </c>
+      <c r="K29" s="3"/>
+      <c r="L29" s="3"/>
+      <c r="M29" s="3"/>
+      <c r="N29" s="3"/>
+      <c r="O29" s="2" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="30" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>990</v>
+      </c>
+      <c r="B30" t="s">
+        <v>991</v>
+      </c>
+      <c r="C30" t="s">
+        <v>190</v>
+      </c>
+      <c r="D30" s="2" t="s">
+        <v>263</v>
+      </c>
+      <c r="E30" s="3">
+        <v>4.24</v>
+      </c>
+      <c r="F30" s="4">
+        <v>105.98</v>
+      </c>
+      <c r="G30" s="3"/>
+      <c r="H30" s="3"/>
+      <c r="I30" s="3">
+        <v>0</v>
+      </c>
+      <c r="J30" s="3">
+        <v>0</v>
+      </c>
+      <c r="K30" s="3"/>
+      <c r="L30" s="3"/>
+      <c r="M30" s="3"/>
+      <c r="N30" s="3"/>
+      <c r="O30" s="2" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="31" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>990</v>
+      </c>
+      <c r="B31" t="s">
+        <v>991</v>
+      </c>
+      <c r="C31" t="s">
+        <v>190</v>
+      </c>
+      <c r="D31" s="2" t="s">
+        <v>273</v>
+      </c>
+      <c r="E31" s="3">
+        <v>4.47</v>
+      </c>
+      <c r="F31" s="4">
+        <v>731.31</v>
+      </c>
+      <c r="G31" s="3"/>
+      <c r="H31" s="3"/>
+      <c r="I31" s="3">
+        <v>6.13</v>
+      </c>
+      <c r="J31" s="3">
+        <v>3.98</v>
+      </c>
+      <c r="K31" s="3"/>
+      <c r="L31" s="3"/>
+      <c r="M31" s="3"/>
+      <c r="N31" s="3"/>
+      <c r="O31" s="2" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="32" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>104</v>
+      </c>
+      <c r="B32" t="s">
+        <v>989</v>
+      </c>
+      <c r="C32" t="s">
+        <v>104</v>
+      </c>
+      <c r="D32" s="2" t="s">
+        <v>280</v>
+      </c>
+      <c r="E32" s="3">
+        <v>4.67</v>
+      </c>
+      <c r="F32" s="4">
+        <v>4.77</v>
+      </c>
+      <c r="G32" s="3"/>
+      <c r="H32" s="3"/>
+      <c r="I32" s="3">
+        <v>2.9</v>
+      </c>
+      <c r="J32" s="3">
+        <v>0.81</v>
+      </c>
+      <c r="K32" s="3"/>
+      <c r="L32" s="3"/>
+      <c r="M32" s="3"/>
+      <c r="N32" s="3"/>
+      <c r="O32" s="2" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="33" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>990</v>
+      </c>
+      <c r="B33" t="s">
+        <v>991</v>
+      </c>
+      <c r="C33" t="s">
+        <v>190</v>
+      </c>
+      <c r="D33" s="2" t="s">
+        <v>284</v>
+      </c>
+      <c r="E33" s="3">
+        <v>4.91</v>
+      </c>
+      <c r="F33" s="4">
+        <v>130.74</v>
+      </c>
+      <c r="G33" s="3"/>
+      <c r="H33" s="3"/>
+      <c r="I33" s="3">
+        <v>8.85</v>
+      </c>
+      <c r="J33" s="3">
+        <v>7.72</v>
+      </c>
+      <c r="K33" s="3"/>
+      <c r="L33" s="3"/>
+      <c r="M33" s="3"/>
+      <c r="N33" s="3"/>
+      <c r="O33" s="2" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="34" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>990</v>
+      </c>
+      <c r="B34" t="s">
+        <v>991</v>
+      </c>
+      <c r="C34" t="s">
+        <v>190</v>
+      </c>
+      <c r="D34" s="2" t="s">
+        <v>290</v>
+      </c>
+      <c r="E34" s="3">
+        <v>5</v>
+      </c>
+      <c r="F34" s="4">
+        <v>106.09</v>
+      </c>
+      <c r="G34" s="3"/>
+      <c r="H34" s="3"/>
+      <c r="I34" s="3">
+        <v>-7.38</v>
+      </c>
+      <c r="J34" s="3">
+        <v>-5.54</v>
+      </c>
+      <c r="K34" s="3"/>
+      <c r="L34" s="3"/>
+      <c r="M34" s="3"/>
+      <c r="N34" s="3"/>
+      <c r="O34" s="2" t="s">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="35" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>992</v>
+      </c>
+      <c r="B35" t="s">
+        <v>989</v>
+      </c>
+      <c r="C35" t="s">
+        <v>158</v>
+      </c>
+      <c r="D35" s="2" t="s">
+        <v>292</v>
+      </c>
+      <c r="E35" s="3">
+        <v>5.08</v>
+      </c>
+      <c r="F35" s="4">
+        <v>972.83</v>
+      </c>
+      <c r="G35" s="3"/>
+      <c r="H35" s="3"/>
+      <c r="I35" s="3">
+        <v>1.97</v>
+      </c>
+      <c r="J35" s="3">
+        <v>0.55</v>
+      </c>
+      <c r="K35" s="3"/>
+      <c r="L35" s="3"/>
+      <c r="M35" s="3"/>
+      <c r="N35" s="3"/>
+      <c r="O35" s="2" t="s">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="36" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>990</v>
+      </c>
+      <c r="B36" t="s">
+        <v>991</v>
+      </c>
+      <c r="C36" t="s">
+        <v>190</v>
+      </c>
+      <c r="D36" s="2" t="s">
+        <v>294</v>
+      </c>
+      <c r="E36" s="3">
+        <v>5.1</v>
+      </c>
+      <c r="F36" s="4">
+        <v>72.56</v>
+      </c>
+      <c r="G36" s="3"/>
+      <c r="H36" s="3"/>
+      <c r="I36" s="3">
+        <v>0.74</v>
+      </c>
+      <c r="J36" s="3">
+        <v>0.57</v>
+      </c>
+      <c r="K36" s="3"/>
+      <c r="L36" s="3"/>
+      <c r="M36" s="3"/>
+      <c r="N36" s="3"/>
+      <c r="O36" s="2" t="s">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="37" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>24</v>
+      </c>
+      <c r="B37" t="s">
+        <v>989</v>
+      </c>
+      <c r="C37" t="s">
+        <v>24</v>
+      </c>
+      <c r="D37" s="2" t="s">
+        <v>319</v>
+      </c>
+      <c r="E37" s="3">
+        <v>5.6</v>
+      </c>
+      <c r="F37" s="4">
+        <v>28.06</v>
+      </c>
+      <c r="G37" s="3"/>
+      <c r="H37" s="3"/>
+      <c r="I37" s="3">
+        <v>0</v>
+      </c>
+      <c r="J37" s="3">
+        <v>0</v>
+      </c>
+      <c r="K37" s="3"/>
+      <c r="L37" s="3"/>
+      <c r="M37" s="3"/>
+      <c r="N37" s="3"/>
+      <c r="O37" s="2" t="s">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="38" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>24</v>
+      </c>
+      <c r="B38" t="s">
+        <v>989</v>
+      </c>
+      <c r="C38" t="s">
+        <v>24</v>
+      </c>
+      <c r="D38" s="2" t="s">
+        <v>334</v>
+      </c>
+      <c r="E38" s="3">
+        <v>5.71</v>
+      </c>
+      <c r="F38" s="4">
+        <v>47.34</v>
+      </c>
+      <c r="G38" s="3"/>
+      <c r="H38" s="3"/>
+      <c r="I38" s="3">
+        <v>0</v>
+      </c>
+      <c r="J38" s="3">
+        <v>0</v>
+      </c>
+      <c r="K38" s="3"/>
+      <c r="L38" s="3"/>
+      <c r="M38" s="3"/>
+      <c r="N38" s="3"/>
+      <c r="O38" s="2" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="39" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>24</v>
+      </c>
+      <c r="B39" t="s">
+        <v>989</v>
+      </c>
+      <c r="C39" t="s">
+        <v>24</v>
+      </c>
+      <c r="D39" s="2" t="s">
+        <v>338</v>
+      </c>
+      <c r="E39" s="3">
+        <v>5.8</v>
+      </c>
+      <c r="F39" s="4">
+        <v>142.64</v>
+      </c>
+      <c r="G39" s="3"/>
+      <c r="H39" s="3"/>
+      <c r="I39" s="3">
+        <v>1.21</v>
+      </c>
+      <c r="J39" s="3">
+        <v>0.96</v>
+      </c>
+      <c r="K39" s="3"/>
+      <c r="L39" s="3"/>
+      <c r="M39" s="3"/>
+      <c r="N39" s="3"/>
+      <c r="O39" s="2" t="s">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="40" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>24</v>
+      </c>
+      <c r="B40" t="s">
+        <v>989</v>
+      </c>
+      <c r="C40" t="s">
+        <v>24</v>
+      </c>
+      <c r="D40" s="2" t="s">
+        <v>359</v>
+      </c>
+      <c r="E40" s="3">
+        <v>6.19</v>
+      </c>
+      <c r="F40" s="4">
+        <v>38.22</v>
+      </c>
+      <c r="G40" s="3"/>
+      <c r="H40" s="3"/>
+      <c r="I40" s="3">
+        <v>0</v>
+      </c>
+      <c r="J40" s="3">
+        <v>0</v>
+      </c>
+      <c r="K40" s="3"/>
+      <c r="L40" s="3"/>
+      <c r="M40" s="3"/>
+      <c r="N40" s="3"/>
+      <c r="O40" s="2" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="41" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>990</v>
+      </c>
+      <c r="B41" t="s">
+        <v>991</v>
+      </c>
+      <c r="C41" t="s">
+        <v>46</v>
+      </c>
+      <c r="D41" s="2" t="s">
+        <v>365</v>
+      </c>
+      <c r="E41" s="3">
+        <v>6.3</v>
+      </c>
+      <c r="F41" s="4">
+        <v>3.71</v>
+      </c>
+      <c r="G41" s="3"/>
+      <c r="H41" s="3"/>
+      <c r="I41" s="3">
+        <v>0</v>
+      </c>
+      <c r="J41" s="3">
+        <v>0</v>
+      </c>
+      <c r="K41" s="3"/>
+      <c r="L41" s="3"/>
+      <c r="M41" s="3"/>
+      <c r="N41" s="3"/>
+      <c r="O41" s="2" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="42" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>990</v>
+      </c>
+      <c r="B42" t="s">
+        <v>997</v>
+      </c>
+      <c r="C42" t="s">
+        <v>72</v>
+      </c>
+      <c r="D42" s="2" t="s">
+        <v>380</v>
+      </c>
+      <c r="E42" s="3">
+        <v>6.5</v>
+      </c>
+      <c r="F42" s="4">
+        <v>12.04</v>
+      </c>
+      <c r="G42" s="3"/>
+      <c r="H42" s="3"/>
+      <c r="I42" s="3">
+        <v>2.52</v>
+      </c>
+      <c r="J42" s="3">
+        <v>1.11</v>
+      </c>
+      <c r="K42" s="3"/>
+      <c r="L42" s="3"/>
+      <c r="M42" s="3"/>
+      <c r="N42" s="3"/>
+      <c r="O42" s="2" t="s">
+        <v>381</v>
+      </c>
+    </row>
+    <row r="43" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>992</v>
+      </c>
+      <c r="B43" t="s">
+        <v>989</v>
+      </c>
+      <c r="C43" t="s">
+        <v>51</v>
+      </c>
+      <c r="D43" s="2" t="s">
+        <v>382</v>
+      </c>
+      <c r="E43" s="3">
+        <v>6.5</v>
+      </c>
+      <c r="F43" s="4">
+        <v>302.78</v>
+      </c>
+      <c r="G43" s="3"/>
+      <c r="H43" s="3"/>
+      <c r="I43" s="3">
+        <v>20.35</v>
+      </c>
+      <c r="J43" s="3">
+        <v>20.26</v>
+      </c>
+      <c r="K43" s="3"/>
+      <c r="L43" s="3"/>
+      <c r="M43" s="3"/>
+      <c r="N43" s="3"/>
+      <c r="O43" s="2" t="s">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="44" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>990</v>
+      </c>
+      <c r="B44" t="s">
+        <v>991</v>
+      </c>
+      <c r="C44" t="s">
+        <v>190</v>
+      </c>
+      <c r="D44" s="2" t="s">
+        <v>384</v>
+      </c>
+      <c r="E44" s="3">
+        <v>6.5</v>
+      </c>
+      <c r="F44" s="4">
+        <v>57.16</v>
+      </c>
+      <c r="G44" s="3"/>
+      <c r="H44" s="3"/>
+      <c r="I44" s="3">
+        <v>0</v>
+      </c>
+      <c r="J44" s="3">
+        <v>0</v>
+      </c>
+      <c r="K44" s="3"/>
+      <c r="L44" s="3"/>
+      <c r="M44" s="3"/>
+      <c r="N44" s="3"/>
+      <c r="O44" s="2" t="s">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="45" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>992</v>
+      </c>
+      <c r="B45" t="s">
+        <v>989</v>
+      </c>
+      <c r="C45" t="s">
+        <v>51</v>
+      </c>
+      <c r="D45" s="2" t="s">
+        <v>390</v>
+      </c>
+      <c r="E45" s="3">
+        <v>6.57</v>
+      </c>
+      <c r="F45" s="4">
+        <v>258.79</v>
+      </c>
+      <c r="G45" s="3"/>
+      <c r="H45" s="3"/>
+      <c r="I45" s="3">
+        <v>18.26</v>
+      </c>
+      <c r="J45" s="3">
+        <v>13.88</v>
+      </c>
+      <c r="K45" s="3"/>
+      <c r="L45" s="3"/>
+      <c r="M45" s="3"/>
+      <c r="N45" s="3"/>
+      <c r="O45" s="2" t="s">
+        <v>391</v>
+      </c>
+    </row>
+    <row r="46" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>404</v>
+      </c>
+      <c r="B46" t="s">
+        <v>989</v>
+      </c>
+      <c r="C46" t="s">
+        <v>404</v>
+      </c>
+      <c r="D46" s="2" t="s">
+        <v>405</v>
+      </c>
+      <c r="E46" s="3">
+        <v>6.74</v>
+      </c>
+      <c r="F46" s="4">
+        <v>3619.45</v>
+      </c>
+      <c r="G46" s="3"/>
+      <c r="H46" s="3"/>
+      <c r="I46" s="3">
+        <v>4.21</v>
+      </c>
+      <c r="J46" s="3">
+        <v>0.61</v>
+      </c>
+      <c r="K46" s="3"/>
+      <c r="L46" s="3"/>
+      <c r="M46" s="3"/>
+      <c r="N46" s="3"/>
+      <c r="O46" s="2" t="s">
+        <v>406</v>
+      </c>
+    </row>
+    <row r="47" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>404</v>
+      </c>
+      <c r="B47" t="s">
+        <v>989</v>
+      </c>
+      <c r="C47" t="s">
+        <v>404</v>
+      </c>
+      <c r="D47" s="2" t="s">
+        <v>407</v>
+      </c>
+      <c r="E47" s="3">
+        <v>6.8</v>
+      </c>
+      <c r="F47" s="4">
+        <v>662.18</v>
+      </c>
+      <c r="G47" s="3"/>
+      <c r="H47" s="3"/>
+      <c r="I47" s="3">
+        <v>2.49</v>
+      </c>
+      <c r="J47" s="3">
+        <v>0.44</v>
+      </c>
+      <c r="K47" s="3"/>
+      <c r="L47" s="3"/>
+      <c r="M47" s="3"/>
+      <c r="N47" s="3"/>
+      <c r="O47" s="2" t="s">
+        <v>408</v>
+      </c>
+    </row>
+    <row r="48" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>992</v>
+      </c>
+      <c r="B48" t="s">
+        <v>989</v>
+      </c>
+      <c r="C48" t="s">
+        <v>51</v>
+      </c>
+      <c r="D48" s="2" t="s">
+        <v>411</v>
+      </c>
+      <c r="E48" s="3">
+        <v>6.8</v>
+      </c>
+      <c r="F48" s="4">
+        <v>116.67</v>
+      </c>
+      <c r="G48" s="3"/>
+      <c r="H48" s="3"/>
+      <c r="I48" s="3">
+        <v>2.45</v>
+      </c>
+      <c r="J48" s="3">
+        <v>-23.09</v>
+      </c>
+      <c r="K48" s="3"/>
+      <c r="L48" s="3"/>
+      <c r="M48" s="3"/>
+      <c r="N48" s="3"/>
+      <c r="O48" s="2" t="s">
+        <v>412</v>
+      </c>
+    </row>
+    <row r="49" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>104</v>
+      </c>
+      <c r="B49" t="s">
+        <v>989</v>
+      </c>
+      <c r="C49" t="s">
+        <v>104</v>
+      </c>
+      <c r="D49" s="2" t="s">
+        <v>419</v>
+      </c>
+      <c r="E49" s="3">
+        <v>6.89</v>
+      </c>
+      <c r="F49" s="4">
+        <v>5.95</v>
+      </c>
+      <c r="G49" s="3"/>
+      <c r="H49" s="3"/>
+      <c r="I49" s="3">
+        <v>2.74</v>
+      </c>
+      <c r="J49" s="3">
+        <v>3.08</v>
+      </c>
+      <c r="K49" s="3"/>
+      <c r="L49" s="3"/>
+      <c r="M49" s="3"/>
+      <c r="N49" s="3"/>
+      <c r="O49" s="2" t="s">
+        <v>420</v>
+      </c>
+    </row>
+    <row r="50" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>992</v>
+      </c>
+      <c r="B50" t="s">
+        <v>989</v>
+      </c>
+      <c r="C50" t="s">
+        <v>51</v>
+      </c>
+      <c r="D50" s="2" t="s">
+        <v>443</v>
+      </c>
+      <c r="E50" s="3">
+        <v>7.31</v>
+      </c>
+      <c r="F50" s="4">
+        <v>197.06</v>
+      </c>
+      <c r="G50" s="3"/>
+      <c r="H50" s="3"/>
+      <c r="I50" s="3">
+        <v>14.57</v>
+      </c>
+      <c r="J50" s="3">
+        <v>11.56</v>
+      </c>
+      <c r="K50" s="3"/>
+      <c r="L50" s="3"/>
+      <c r="M50" s="3"/>
+      <c r="N50" s="3"/>
+      <c r="O50" s="2" t="s">
+        <v>444</v>
+      </c>
+    </row>
+    <row r="51" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>994</v>
+      </c>
+      <c r="B51" t="s">
+        <v>989</v>
+      </c>
+      <c r="C51" t="s">
+        <v>473</v>
+      </c>
+      <c r="D51" s="2" t="s">
+        <v>474</v>
+      </c>
+      <c r="E51" s="3">
+        <v>7.79</v>
+      </c>
+      <c r="F51" s="4">
+        <v>1245.23</v>
+      </c>
+      <c r="G51" s="3"/>
+      <c r="H51" s="3"/>
+      <c r="I51" s="3">
+        <v>20.91</v>
+      </c>
+      <c r="J51" s="3">
+        <v>38.89</v>
+      </c>
+      <c r="K51" s="3"/>
+      <c r="L51" s="3"/>
+      <c r="M51" s="3"/>
+      <c r="N51" s="3"/>
+      <c r="O51" s="2" t="s">
+        <v>475</v>
+      </c>
+    </row>
+    <row r="52" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>992</v>
+      </c>
+      <c r="B52" t="s">
+        <v>989</v>
+      </c>
+      <c r="C52" t="s">
+        <v>51</v>
+      </c>
+      <c r="D52" s="2" t="s">
+        <v>476</v>
+      </c>
+      <c r="E52" s="3">
+        <v>7.79</v>
+      </c>
+      <c r="F52" s="4">
+        <v>120.75</v>
+      </c>
+      <c r="G52" s="3"/>
+      <c r="H52" s="3"/>
+      <c r="I52" s="3">
+        <v>20.91</v>
+      </c>
+      <c r="J52" s="3">
+        <v>23.35</v>
+      </c>
+      <c r="K52" s="3"/>
+      <c r="L52" s="3"/>
+      <c r="M52" s="3"/>
+      <c r="N52" s="3"/>
+      <c r="O52" s="2" t="s">
+        <v>477</v>
+      </c>
+    </row>
+    <row r="53" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>990</v>
+      </c>
+      <c r="B53" t="s">
+        <v>991</v>
+      </c>
+      <c r="C53" t="s">
+        <v>46</v>
+      </c>
+      <c r="D53" s="2" t="s">
+        <v>497</v>
+      </c>
+      <c r="E53" s="3">
+        <v>8.1</v>
+      </c>
+      <c r="F53" s="4">
+        <v>4.33</v>
+      </c>
+      <c r="G53" s="3"/>
+      <c r="H53" s="3"/>
+      <c r="I53" s="3">
+        <v>0</v>
+      </c>
+      <c r="J53" s="3">
+        <v>0</v>
+      </c>
+      <c r="K53" s="3"/>
+      <c r="L53" s="3"/>
+      <c r="M53" s="3"/>
+      <c r="N53" s="3"/>
+      <c r="O53" s="2" t="s">
+        <v>498</v>
+      </c>
+    </row>
+    <row r="54" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>24</v>
+      </c>
+      <c r="B54" t="s">
+        <v>989</v>
+      </c>
+      <c r="C54" t="s">
+        <v>24</v>
+      </c>
+      <c r="D54" s="2" t="s">
+        <v>505</v>
+      </c>
+      <c r="E54" s="3">
+        <v>8.18</v>
+      </c>
+      <c r="F54" s="4">
+        <v>35.32</v>
+      </c>
+      <c r="G54" s="3"/>
+      <c r="H54" s="3"/>
+      <c r="I54" s="3">
+        <v>0</v>
+      </c>
+      <c r="J54" s="3">
+        <v>0</v>
+      </c>
+      <c r="K54" s="3"/>
+      <c r="L54" s="3"/>
+      <c r="M54" s="3"/>
+      <c r="N54" s="3"/>
+      <c r="O54" s="2" t="s">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="55" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>24</v>
+      </c>
+      <c r="B55" t="s">
+        <v>989</v>
+      </c>
+      <c r="C55" t="s">
+        <v>24</v>
+      </c>
+      <c r="D55" s="2" t="s">
+        <v>510</v>
+      </c>
+      <c r="E55" s="3">
+        <v>8.38</v>
+      </c>
+      <c r="F55" s="4">
+        <v>109.33</v>
+      </c>
+      <c r="G55" s="3"/>
+      <c r="H55" s="3"/>
+      <c r="I55" s="3">
+        <v>4.92</v>
+      </c>
+      <c r="J55" s="3">
+        <v>1.52</v>
+      </c>
+      <c r="K55" s="3"/>
+      <c r="L55" s="3"/>
+      <c r="M55" s="3"/>
+      <c r="N55" s="3"/>
+      <c r="O55" s="2" t="s">
+        <v>511</v>
+      </c>
+    </row>
+    <row r="56" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>404</v>
+      </c>
+      <c r="B56" t="s">
+        <v>989</v>
+      </c>
+      <c r="C56" t="s">
+        <v>404</v>
+      </c>
+      <c r="D56" s="2" t="s">
+        <v>512</v>
+      </c>
+      <c r="E56" s="3">
+        <v>8.44</v>
+      </c>
+      <c r="F56" s="4">
+        <v>135.89</v>
+      </c>
+      <c r="G56" s="3"/>
+      <c r="H56" s="3"/>
+      <c r="I56" s="3">
+        <v>1.44</v>
+      </c>
+      <c r="J56" s="3">
+        <v>0.09</v>
+      </c>
+      <c r="K56" s="3"/>
+      <c r="L56" s="3"/>
+      <c r="M56" s="3"/>
+      <c r="N56" s="3"/>
+      <c r="O56" s="2" t="s">
+        <v>513</v>
+      </c>
+    </row>
+    <row r="57" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>990</v>
+      </c>
+      <c r="B57" t="s">
+        <v>991</v>
+      </c>
+      <c r="C57" t="s">
+        <v>46</v>
+      </c>
+      <c r="D57" s="2" t="s">
+        <v>521</v>
+      </c>
+      <c r="E57" s="3">
+        <v>8.6</v>
+      </c>
+      <c r="F57" s="4">
+        <v>4.26</v>
+      </c>
+      <c r="G57" s="3"/>
+      <c r="H57" s="3"/>
+      <c r="I57" s="3">
+        <v>0</v>
+      </c>
+      <c r="J57" s="3">
+        <v>0</v>
+      </c>
+      <c r="K57" s="3"/>
+      <c r="L57" s="3"/>
+      <c r="M57" s="3"/>
+      <c r="N57" s="3"/>
+      <c r="O57" s="2" t="s">
+        <v>522</v>
+      </c>
+    </row>
+    <row r="58" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>404</v>
+      </c>
+      <c r="B58" t="s">
+        <v>989</v>
+      </c>
+      <c r="C58" t="s">
+        <v>404</v>
+      </c>
+      <c r="D58" s="2" t="s">
+        <v>527</v>
+      </c>
+      <c r="E58" s="3">
+        <v>8.77</v>
+      </c>
+      <c r="F58" s="4">
+        <v>1028.75</v>
+      </c>
+      <c r="G58" s="3"/>
+      <c r="H58" s="3"/>
+      <c r="I58" s="3">
+        <v>0</v>
+      </c>
+      <c r="J58" s="3">
+        <v>0</v>
+      </c>
+      <c r="K58" s="3"/>
+      <c r="L58" s="3"/>
+      <c r="M58" s="3"/>
+      <c r="N58" s="3"/>
+      <c r="O58" s="2" t="s">
+        <v>528</v>
+      </c>
+    </row>
+    <row r="59" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>990</v>
+      </c>
+      <c r="B59" t="s">
+        <v>991</v>
+      </c>
+      <c r="C59" t="s">
+        <v>190</v>
+      </c>
+      <c r="D59" s="2" t="s">
+        <v>533</v>
+      </c>
+      <c r="E59" s="3">
+        <v>8.87</v>
+      </c>
+      <c r="F59" s="4">
+        <v>38.81</v>
+      </c>
+      <c r="G59" s="3"/>
+      <c r="H59" s="3"/>
+      <c r="I59" s="3">
+        <v>15.01</v>
+      </c>
+      <c r="J59" s="3">
+        <v>13.21</v>
+      </c>
+      <c r="K59" s="3"/>
+      <c r="L59" s="3"/>
+      <c r="M59" s="3"/>
+      <c r="N59" s="3"/>
+      <c r="O59" s="2" t="s">
+        <v>534</v>
+      </c>
+    </row>
+    <row r="60" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>990</v>
+      </c>
+      <c r="B60" t="s">
+        <v>996</v>
+      </c>
+      <c r="C60" t="s">
+        <v>220</v>
+      </c>
+      <c r="D60" s="2" t="s">
+        <v>545</v>
+      </c>
+      <c r="E60" s="3">
+        <v>9.04</v>
+      </c>
+      <c r="F60" s="4">
+        <v>178.44</v>
+      </c>
+      <c r="G60" s="3"/>
+      <c r="H60" s="3"/>
+      <c r="I60" s="3">
+        <v>20.19</v>
+      </c>
+      <c r="J60" s="3">
+        <v>20.78</v>
+      </c>
+      <c r="K60" s="3"/>
+      <c r="L60" s="3"/>
+      <c r="M60" s="3"/>
+      <c r="N60" s="3"/>
+      <c r="O60" s="2" t="s">
+        <v>546</v>
+      </c>
+    </row>
+    <row r="61" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>104</v>
+      </c>
+      <c r="B61" t="s">
+        <v>989</v>
+      </c>
+      <c r="C61" t="s">
+        <v>104</v>
+      </c>
+      <c r="D61" s="2" t="s">
+        <v>574</v>
+      </c>
+      <c r="E61" s="3">
+        <v>9.67</v>
+      </c>
+      <c r="F61" s="4">
+        <v>10.15</v>
+      </c>
+      <c r="G61" s="3"/>
+      <c r="H61" s="3"/>
+      <c r="I61" s="3">
+        <v>0.19</v>
+      </c>
+      <c r="J61" s="3">
+        <v>0.13</v>
+      </c>
+      <c r="K61" s="3"/>
+      <c r="L61" s="3"/>
+      <c r="M61" s="3"/>
+      <c r="N61" s="3"/>
+      <c r="O61" s="2" t="s">
+        <v>575</v>
+      </c>
+    </row>
+    <row r="62" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>24</v>
+      </c>
+      <c r="B62" t="s">
+        <v>989</v>
+      </c>
+      <c r="C62" t="s">
+        <v>24</v>
+      </c>
+      <c r="D62" s="2" t="s">
+        <v>578</v>
+      </c>
+      <c r="E62" s="3">
+        <v>9.8</v>
+      </c>
+      <c r="F62" s="4">
+        <v>238.09</v>
+      </c>
+      <c r="G62" s="3"/>
+      <c r="H62" s="3"/>
+      <c r="I62" s="3">
+        <v>9.52</v>
+      </c>
+      <c r="J62" s="3">
+        <v>8.01</v>
+      </c>
+      <c r="K62" s="3"/>
+      <c r="L62" s="3"/>
+      <c r="M62" s="3"/>
+      <c r="N62" s="3"/>
+      <c r="O62" s="2" t="s">
+        <v>579</v>
+      </c>
+    </row>
+    <row r="63" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>990</v>
+      </c>
+      <c r="B63" t="s">
+        <v>991</v>
+      </c>
+      <c r="C63" t="s">
+        <v>46</v>
+      </c>
+      <c r="D63" s="2" t="s">
+        <v>582</v>
+      </c>
+      <c r="E63" s="3">
+        <v>9.95</v>
+      </c>
+      <c r="F63" s="4">
+        <v>5.25</v>
+      </c>
+      <c r="G63" s="3"/>
+      <c r="H63" s="3"/>
+      <c r="I63" s="3">
+        <v>8.6</v>
+      </c>
+      <c r="J63" s="3">
+        <v>9.78</v>
+      </c>
+      <c r="K63" s="3"/>
+      <c r="L63" s="3"/>
+      <c r="M63" s="3"/>
+      <c r="N63" s="3"/>
+      <c r="O63" s="2" t="s">
+        <v>583</v>
+      </c>
+    </row>
+    <row r="64" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
+        <v>24</v>
+      </c>
+      <c r="B64" t="s">
+        <v>989</v>
+      </c>
+      <c r="C64" t="s">
+        <v>24</v>
+      </c>
+      <c r="D64" s="2" t="s">
+        <v>584</v>
+      </c>
+      <c r="E64" s="3">
+        <v>10</v>
+      </c>
+      <c r="F64" s="4">
+        <v>33</v>
+      </c>
+      <c r="G64" s="3"/>
+      <c r="H64" s="3"/>
+      <c r="I64" s="3">
+        <v>15.77</v>
+      </c>
+      <c r="J64" s="3">
+        <v>11.09</v>
+      </c>
+      <c r="K64" s="3"/>
+      <c r="L64" s="3"/>
+      <c r="M64" s="3"/>
+      <c r="N64" s="3"/>
+      <c r="O64" s="2" t="s">
+        <v>585</v>
+      </c>
+    </row>
+    <row r="65" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
+        <v>990</v>
+      </c>
+      <c r="B65" t="s">
+        <v>991</v>
+      </c>
+      <c r="C65" t="s">
+        <v>190</v>
+      </c>
+      <c r="D65" s="2" t="s">
+        <v>586</v>
+      </c>
+      <c r="E65" s="3">
+        <v>10</v>
+      </c>
+      <c r="F65" s="4">
+        <v>131.14</v>
+      </c>
+      <c r="G65" s="3"/>
+      <c r="H65" s="3"/>
+      <c r="I65" s="3">
+        <v>14.38</v>
+      </c>
+      <c r="J65" s="3">
+        <v>10.51</v>
+      </c>
+      <c r="K65" s="3"/>
+      <c r="L65" s="3"/>
+      <c r="M65" s="3"/>
+      <c r="N65" s="3"/>
+      <c r="O65" s="2" t="s">
+        <v>587</v>
+      </c>
+    </row>
+    <row r="66" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
+        <v>104</v>
+      </c>
+      <c r="B66" t="s">
+        <v>989</v>
+      </c>
+      <c r="C66" t="s">
+        <v>104</v>
+      </c>
+      <c r="D66" s="2" t="s">
+        <v>590</v>
+      </c>
+      <c r="E66" s="3">
+        <v>10.12</v>
+      </c>
+      <c r="F66" s="4">
+        <v>7.08</v>
+      </c>
+      <c r="G66" s="3"/>
+      <c r="H66" s="3"/>
+      <c r="I66" s="3">
+        <v>0</v>
+      </c>
+      <c r="J66" s="3">
+        <v>0</v>
+      </c>
+      <c r="K66" s="3"/>
+      <c r="L66" s="3"/>
+      <c r="M66" s="3"/>
+      <c r="N66" s="3"/>
+      <c r="O66" s="2" t="s">
+        <v>591</v>
+      </c>
+    </row>
+    <row r="67" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
+        <v>24</v>
+      </c>
+      <c r="B67" t="s">
+        <v>989</v>
+      </c>
+      <c r="C67" t="s">
+        <v>24</v>
+      </c>
+      <c r="D67" s="2" t="s">
+        <v>592</v>
+      </c>
+      <c r="E67" s="3">
+        <v>10.23</v>
+      </c>
+      <c r="F67" s="4">
+        <v>198.73</v>
+      </c>
+      <c r="G67" s="3"/>
+      <c r="H67" s="3"/>
+      <c r="I67" s="3">
+        <v>0.05</v>
+      </c>
+      <c r="J67" s="3">
+        <v>-31.28</v>
+      </c>
+      <c r="K67" s="3"/>
+      <c r="L67" s="3"/>
+      <c r="M67" s="3"/>
+      <c r="N67" s="3"/>
+      <c r="O67" s="2" t="s">
+        <v>593</v>
+      </c>
+    </row>
+    <row r="68" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A68" t="s">
+        <v>992</v>
+      </c>
+      <c r="B68" t="s">
+        <v>989</v>
+      </c>
+      <c r="C68" t="s">
+        <v>51</v>
+      </c>
+      <c r="D68" s="2" t="s">
+        <v>632</v>
+      </c>
+      <c r="E68" s="3">
+        <v>11.22</v>
+      </c>
+      <c r="F68" s="4">
+        <v>105.19</v>
+      </c>
+      <c r="G68" s="3"/>
+      <c r="H68" s="3"/>
+      <c r="I68" s="3">
+        <v>6.88</v>
+      </c>
+      <c r="J68" s="3">
+        <v>4.21</v>
+      </c>
+      <c r="K68" s="3"/>
+      <c r="L68" s="3"/>
+      <c r="M68" s="3"/>
+      <c r="N68" s="3"/>
+      <c r="O68" s="2" t="s">
+        <v>633</v>
+      </c>
+    </row>
+    <row r="69" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A69" t="s">
+        <v>990</v>
+      </c>
+      <c r="B69" t="s">
+        <v>991</v>
+      </c>
+      <c r="C69" t="s">
+        <v>190</v>
+      </c>
+      <c r="D69" s="2" t="s">
+        <v>636</v>
+      </c>
+      <c r="E69" s="3">
+        <v>11.22</v>
+      </c>
+      <c r="F69" s="4">
+        <v>1431.13</v>
+      </c>
+      <c r="G69" s="3"/>
+      <c r="H69" s="3"/>
+      <c r="I69" s="3">
+        <v>8.8</v>
+      </c>
+      <c r="J69" s="3">
+        <v>2.65</v>
+      </c>
+      <c r="K69" s="3"/>
+      <c r="L69" s="3"/>
+      <c r="M69" s="3"/>
+      <c r="N69" s="3"/>
+      <c r="O69" s="2" t="s">
+        <v>637</v>
+      </c>
+    </row>
+    <row r="70" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
+        <v>104</v>
+      </c>
+      <c r="B70" t="s">
+        <v>989</v>
+      </c>
+      <c r="C70" t="s">
+        <v>104</v>
+      </c>
+      <c r="D70" s="2" t="s">
+        <v>657</v>
+      </c>
+      <c r="E70" s="3">
+        <v>11.7</v>
+      </c>
+      <c r="F70" s="4">
+        <v>28.96</v>
+      </c>
+      <c r="G70" s="3"/>
+      <c r="H70" s="3"/>
+      <c r="I70" s="3">
+        <v>3.08</v>
+      </c>
+      <c r="J70" s="3">
+        <v>2.11</v>
+      </c>
+      <c r="K70" s="3"/>
+      <c r="L70" s="3"/>
+      <c r="M70" s="3"/>
+      <c r="N70" s="3"/>
+      <c r="O70" s="2" t="s">
+        <v>658</v>
+      </c>
+    </row>
+    <row r="71" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A71" t="s">
+        <v>990</v>
+      </c>
+      <c r="B71" t="s">
+        <v>991</v>
+      </c>
+      <c r="C71" t="s">
+        <v>46</v>
+      </c>
+      <c r="D71" s="2" t="s">
+        <v>659</v>
+      </c>
+      <c r="E71" s="3">
+        <v>11.93</v>
+      </c>
+      <c r="F71" s="4">
+        <v>14.6</v>
+      </c>
+      <c r="G71" s="3"/>
+      <c r="H71" s="3"/>
+      <c r="I71" s="3">
+        <v>-9.63</v>
+      </c>
+      <c r="J71" s="3">
+        <v>-14</v>
+      </c>
+      <c r="K71" s="3"/>
+      <c r="L71" s="3"/>
+      <c r="M71" s="3"/>
+      <c r="N71" s="3"/>
+      <c r="O71" s="2" t="s">
+        <v>660</v>
+      </c>
+    </row>
+    <row r="72" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A72" t="s">
+        <v>104</v>
+      </c>
+      <c r="B72" t="s">
+        <v>989</v>
+      </c>
+      <c r="C72" t="s">
+        <v>104</v>
+      </c>
+      <c r="D72" s="2" t="s">
+        <v>667</v>
+      </c>
+      <c r="E72" s="3">
+        <v>12.15</v>
+      </c>
+      <c r="F72" s="4">
+        <v>12.76</v>
+      </c>
+      <c r="G72" s="3"/>
+      <c r="H72" s="3"/>
+      <c r="I72" s="3">
+        <v>0</v>
+      </c>
+      <c r="J72" s="3">
+        <v>0</v>
+      </c>
+      <c r="K72" s="3"/>
+      <c r="L72" s="3"/>
+      <c r="M72" s="3"/>
+      <c r="N72" s="3"/>
+      <c r="O72" s="2" t="s">
+        <v>668</v>
+      </c>
+    </row>
+    <row r="73" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A73" t="s">
+        <v>998</v>
+      </c>
+      <c r="B73" t="s">
+        <v>989</v>
+      </c>
+      <c r="C73" t="s">
+        <v>669</v>
+      </c>
+      <c r="D73" s="2" t="s">
+        <v>670</v>
+      </c>
+      <c r="E73" s="3">
+        <v>12.19</v>
+      </c>
+      <c r="F73" s="4">
+        <v>1.87</v>
+      </c>
+      <c r="G73" s="3"/>
+      <c r="H73" s="3"/>
+      <c r="I73" s="3">
+        <v>0</v>
+      </c>
+      <c r="J73" s="3">
+        <v>0</v>
+      </c>
+      <c r="K73" s="3"/>
+      <c r="L73" s="3"/>
+      <c r="M73" s="3"/>
+      <c r="N73" s="3"/>
+      <c r="O73" s="2" t="s">
+        <v>671</v>
+      </c>
+    </row>
+    <row r="74" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A74" t="s">
+        <v>990</v>
+      </c>
+      <c r="B74" t="s">
+        <v>991</v>
+      </c>
+      <c r="C74" t="s">
+        <v>190</v>
+      </c>
+      <c r="D74" s="2" t="s">
+        <v>674</v>
+      </c>
+      <c r="E74" s="3">
+        <v>12.29</v>
+      </c>
+      <c r="F74" s="4">
+        <v>110.05</v>
+      </c>
+      <c r="G74" s="3"/>
+      <c r="H74" s="3"/>
+      <c r="I74" s="3">
+        <v>4.92</v>
+      </c>
+      <c r="J74" s="3">
+        <v>9.93</v>
+      </c>
+      <c r="K74" s="3"/>
+      <c r="L74" s="3"/>
+      <c r="M74" s="3"/>
+      <c r="N74" s="3"/>
+      <c r="O74" s="2" t="s">
+        <v>675</v>
+      </c>
+    </row>
+    <row r="75" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A75" t="s">
+        <v>992</v>
+      </c>
+      <c r="B75" t="s">
+        <v>989</v>
+      </c>
+      <c r="C75" t="s">
+        <v>158</v>
+      </c>
+      <c r="D75" s="2" t="s">
+        <v>684</v>
+      </c>
+      <c r="E75" s="3">
+        <v>12.56</v>
+      </c>
+      <c r="F75" s="4">
+        <v>802.32</v>
+      </c>
+      <c r="G75" s="3"/>
+      <c r="H75" s="3"/>
+      <c r="I75" s="3">
+        <v>17.09</v>
+      </c>
+      <c r="J75" s="3">
+        <v>16.8</v>
+      </c>
+      <c r="K75" s="3"/>
+      <c r="L75" s="3"/>
+      <c r="M75" s="3"/>
+      <c r="N75" s="3"/>
+      <c r="O75" s="2" t="s">
+        <v>685</v>
+      </c>
+    </row>
+    <row r="76" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A76" t="s">
+        <v>104</v>
+      </c>
+      <c r="B76" t="s">
+        <v>989</v>
+      </c>
+      <c r="C76" t="s">
+        <v>104</v>
+      </c>
+      <c r="D76" s="2" t="s">
+        <v>688</v>
+      </c>
+      <c r="E76" s="3">
+        <v>12.65</v>
+      </c>
+      <c r="F76" s="4">
+        <v>187.14</v>
+      </c>
+      <c r="G76" s="3"/>
+      <c r="H76" s="3"/>
+      <c r="I76" s="3">
+        <v>0.88</v>
+      </c>
+      <c r="J76" s="3">
+        <v>0.76</v>
+      </c>
+      <c r="K76" s="3"/>
+      <c r="L76" s="3"/>
+      <c r="M76" s="3"/>
+      <c r="N76" s="3"/>
+      <c r="O76" s="2" t="s">
+        <v>689</v>
+      </c>
+    </row>
+    <row r="77" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A77" t="s">
+        <v>104</v>
+      </c>
+      <c r="B77" t="s">
+        <v>989</v>
+      </c>
+      <c r="C77" t="s">
+        <v>104</v>
+      </c>
+      <c r="D77" s="2" t="s">
+        <v>692</v>
+      </c>
+      <c r="E77" s="3">
+        <v>12.7</v>
+      </c>
+      <c r="F77" s="4">
+        <v>25.47</v>
+      </c>
+      <c r="G77" s="3"/>
+      <c r="H77" s="3"/>
+      <c r="I77" s="3">
+        <v>7.07</v>
+      </c>
+      <c r="J77" s="3">
+        <v>5.29</v>
+      </c>
+      <c r="K77" s="3"/>
+      <c r="L77" s="3"/>
+      <c r="M77" s="3"/>
+      <c r="N77" s="3"/>
+      <c r="O77" s="2" t="s">
+        <v>693</v>
+      </c>
+    </row>
+    <row r="78" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A78" t="s">
+        <v>990</v>
+      </c>
+      <c r="B78" t="s">
+        <v>991</v>
+      </c>
+      <c r="C78" t="s">
+        <v>190</v>
+      </c>
+      <c r="D78" s="2" t="s">
+        <v>694</v>
+      </c>
+      <c r="E78" s="3">
+        <v>12.75</v>
+      </c>
+      <c r="F78" s="4">
+        <v>46.08</v>
+      </c>
+      <c r="G78" s="3"/>
+      <c r="H78" s="3"/>
+      <c r="I78" s="3">
+        <v>-2.48</v>
+      </c>
+      <c r="J78" s="3">
+        <v>14.45</v>
+      </c>
+      <c r="K78" s="3"/>
+      <c r="L78" s="3"/>
+      <c r="M78" s="3"/>
+      <c r="N78" s="3"/>
+      <c r="O78" s="2" t="s">
+        <v>695</v>
+      </c>
+    </row>
+    <row r="79" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A79" t="s">
+        <v>992</v>
+      </c>
+      <c r="B79" t="s">
+        <v>989</v>
+      </c>
+      <c r="C79" t="s">
+        <v>51</v>
+      </c>
+      <c r="D79" s="2" t="s">
+        <v>696</v>
+      </c>
+      <c r="E79" s="3">
+        <v>12.78</v>
+      </c>
+      <c r="F79" s="4">
+        <v>158.34</v>
+      </c>
+      <c r="G79" s="3"/>
+      <c r="H79" s="3"/>
+      <c r="I79" s="3">
+        <v>10.5</v>
+      </c>
+      <c r="J79" s="3">
+        <v>7.95</v>
+      </c>
+      <c r="K79" s="3"/>
+      <c r="L79" s="3"/>
+      <c r="M79" s="3"/>
+      <c r="N79" s="3"/>
+      <c r="O79" s="2" t="s">
+        <v>697</v>
+      </c>
+    </row>
+    <row r="80" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A80" t="s">
+        <v>104</v>
+      </c>
+      <c r="B80" t="s">
+        <v>989</v>
+      </c>
+      <c r="C80" t="s">
+        <v>104</v>
+      </c>
+      <c r="D80" s="2" t="s">
+        <v>702</v>
+      </c>
+      <c r="E80" s="3">
+        <v>12.9</v>
+      </c>
+      <c r="F80" s="4">
+        <v>17.93</v>
+      </c>
+      <c r="G80" s="3"/>
+      <c r="H80" s="3"/>
+      <c r="I80" s="3">
+        <v>5.97</v>
+      </c>
+      <c r="J80" s="3">
+        <v>2.58</v>
+      </c>
+      <c r="K80" s="3"/>
+      <c r="L80" s="3"/>
+      <c r="M80" s="3"/>
+      <c r="N80" s="3"/>
+      <c r="O80" s="2" t="s">
+        <v>703</v>
+      </c>
+    </row>
+    <row r="81" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A81" t="s">
+        <v>992</v>
+      </c>
+      <c r="B81" t="s">
+        <v>989</v>
+      </c>
+      <c r="C81" t="s">
+        <v>158</v>
+      </c>
+      <c r="D81" s="2" t="s">
+        <v>737</v>
+      </c>
+      <c r="E81" s="3">
+        <v>13.45</v>
+      </c>
+      <c r="F81" s="4">
+        <v>600.89</v>
+      </c>
+      <c r="G81" s="3"/>
+      <c r="H81" s="3"/>
+      <c r="I81" s="3">
+        <v>4.03</v>
+      </c>
+      <c r="J81" s="3">
+        <v>-2.55</v>
+      </c>
+      <c r="K81" s="3"/>
+      <c r="L81" s="3"/>
+      <c r="M81" s="3"/>
+      <c r="N81" s="3"/>
+      <c r="O81" s="2" t="s">
+        <v>738</v>
+      </c>
+    </row>
+    <row r="82" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A82" t="s">
+        <v>990</v>
+      </c>
+      <c r="B82" t="s">
+        <v>991</v>
+      </c>
+      <c r="C82" t="s">
+        <v>46</v>
+      </c>
+      <c r="D82" s="2" t="s">
+        <v>755</v>
+      </c>
+      <c r="E82" s="3">
+        <v>13.86</v>
+      </c>
+      <c r="F82" s="4">
+        <v>16.56</v>
+      </c>
+      <c r="G82" s="3"/>
+      <c r="H82" s="3"/>
+      <c r="I82" s="3">
+        <v>1.81</v>
+      </c>
+      <c r="J82" s="3">
+        <v>4.24</v>
+      </c>
+      <c r="K82" s="3"/>
+      <c r="L82" s="3"/>
+      <c r="M82" s="3"/>
+      <c r="N82" s="3"/>
+      <c r="O82" s="2" t="s">
+        <v>756</v>
+      </c>
+    </row>
+    <row r="83" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A83" t="s">
+        <v>404</v>
+      </c>
+      <c r="B83" t="s">
+        <v>989</v>
+      </c>
+      <c r="C83" t="s">
+        <v>404</v>
+      </c>
+      <c r="D83" s="2" t="s">
+        <v>757</v>
+      </c>
+      <c r="E83" s="3">
+        <v>13.91</v>
+      </c>
+      <c r="F83" s="4">
+        <v>19.37</v>
+      </c>
+      <c r="G83" s="3"/>
+      <c r="H83" s="3"/>
+      <c r="I83" s="3">
+        <v>0.07</v>
+      </c>
+      <c r="J83" s="3">
+        <v>0.34</v>
+      </c>
+      <c r="K83" s="3"/>
+      <c r="L83" s="3"/>
+      <c r="M83" s="3"/>
+      <c r="N83" s="3"/>
+      <c r="O83" s="2" t="s">
+        <v>758</v>
+      </c>
+    </row>
+    <row r="84" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A84" t="s">
+        <v>990</v>
+      </c>
+      <c r="B84" t="s">
+        <v>991</v>
+      </c>
+      <c r="C84" t="s">
+        <v>46</v>
+      </c>
+      <c r="D84" s="2" t="s">
+        <v>759</v>
+      </c>
+      <c r="E84" s="3">
+        <v>14.12</v>
+      </c>
+      <c r="F84" s="4">
+        <v>19.46</v>
+      </c>
+      <c r="G84" s="3"/>
+      <c r="H84" s="3"/>
+      <c r="I84" s="3">
+        <v>8.38</v>
+      </c>
+      <c r="J84" s="3">
+        <v>8.41</v>
+      </c>
+      <c r="K84" s="3"/>
+      <c r="L84" s="3"/>
+      <c r="M84" s="3"/>
+      <c r="N84" s="3"/>
+      <c r="O84" s="2" t="s">
+        <v>760</v>
+      </c>
+    </row>
+    <row r="85" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A85" t="s">
+        <v>992</v>
+      </c>
+      <c r="B85" t="s">
+        <v>989</v>
+      </c>
+      <c r="C85" t="s">
+        <v>51</v>
+      </c>
+      <c r="D85" s="2" t="s">
+        <v>767</v>
+      </c>
+      <c r="E85" s="3">
+        <v>14.38</v>
+      </c>
+      <c r="F85" s="4">
+        <v>255.28</v>
+      </c>
+      <c r="G85" s="3"/>
+      <c r="H85" s="3"/>
+      <c r="I85" s="3">
+        <v>0</v>
+      </c>
+      <c r="J85" s="3">
+        <v>0</v>
+      </c>
+      <c r="K85" s="3"/>
+      <c r="L85" s="3"/>
+      <c r="M85" s="3"/>
+      <c r="N85" s="3"/>
+      <c r="O85" s="2" t="s">
+        <v>768</v>
+      </c>
+    </row>
+    <row r="86" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A86" t="s">
+        <v>990</v>
+      </c>
+      <c r="B86" t="s">
+        <v>991</v>
+      </c>
+      <c r="C86" t="s">
+        <v>46</v>
+      </c>
+      <c r="D86" s="2" t="s">
+        <v>769</v>
+      </c>
+      <c r="E86" s="3">
+        <v>14.43</v>
+      </c>
+      <c r="F86" s="4">
+        <v>6.86</v>
+      </c>
+      <c r="G86" s="3"/>
+      <c r="H86" s="3"/>
+      <c r="I86" s="3">
+        <v>0</v>
+      </c>
+      <c r="J86" s="3">
+        <v>0</v>
+      </c>
+      <c r="K86" s="3"/>
+      <c r="L86" s="3"/>
+      <c r="M86" s="3"/>
+      <c r="N86" s="3"/>
+      <c r="O86" s="2" t="s">
+        <v>770</v>
+      </c>
+    </row>
+    <row r="87" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A87" t="s">
+        <v>404</v>
+      </c>
+      <c r="B87" t="s">
+        <v>989</v>
+      </c>
+      <c r="C87" t="s">
+        <v>404</v>
+      </c>
+      <c r="D87" s="2" t="s">
+        <v>777</v>
+      </c>
+      <c r="E87" s="3">
+        <v>14.52</v>
+      </c>
+      <c r="F87" s="4">
+        <v>68.97</v>
+      </c>
+      <c r="G87" s="3"/>
+      <c r="H87" s="3"/>
+      <c r="I87" s="3">
+        <v>0</v>
+      </c>
+      <c r="J87" s="3">
+        <v>0</v>
+      </c>
+      <c r="K87" s="3"/>
+      <c r="L87" s="3"/>
+      <c r="M87" s="3"/>
+      <c r="N87" s="3"/>
+      <c r="O87" s="2" t="s">
+        <v>778</v>
+      </c>
+    </row>
+    <row r="88" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A88" t="s">
+        <v>24</v>
+      </c>
+      <c r="B88" t="s">
+        <v>989</v>
+      </c>
+      <c r="C88" t="s">
+        <v>24</v>
+      </c>
+      <c r="D88" s="2" t="s">
+        <v>787</v>
+      </c>
+      <c r="E88" s="3">
+        <v>14.76</v>
+      </c>
+      <c r="F88" s="4">
+        <v>21</v>
+      </c>
+      <c r="G88" s="3"/>
+      <c r="H88" s="3"/>
+      <c r="I88" s="3">
+        <v>2.28</v>
+      </c>
+      <c r="J88" s="3">
+        <v>2.07</v>
+      </c>
+      <c r="K88" s="3"/>
+      <c r="L88" s="3"/>
+      <c r="M88" s="3"/>
+      <c r="N88" s="3"/>
+      <c r="O88" s="2" t="s">
+        <v>788</v>
+      </c>
+    </row>
+    <row r="89" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A89" t="s">
+        <v>404</v>
+      </c>
+      <c r="B89" t="s">
+        <v>989</v>
+      </c>
+      <c r="C89" t="s">
+        <v>404</v>
+      </c>
+      <c r="D89" s="2" t="s">
+        <v>793</v>
+      </c>
+      <c r="E89" s="3">
+        <v>14.8</v>
+      </c>
+      <c r="F89" s="4">
+        <v>10143.12</v>
+      </c>
+      <c r="G89" s="3"/>
+      <c r="H89" s="3"/>
+      <c r="I89" s="3">
+        <v>6.35</v>
+      </c>
+      <c r="J89" s="3">
+        <v>3.21</v>
+      </c>
+      <c r="K89" s="3"/>
+      <c r="L89" s="3"/>
+      <c r="M89" s="3"/>
+      <c r="N89" s="3"/>
+      <c r="O89" s="2" t="s">
+        <v>794</v>
+      </c>
+    </row>
+    <row r="90" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A90" t="s">
+        <v>104</v>
+      </c>
+      <c r="B90" t="s">
+        <v>989</v>
+      </c>
+      <c r="C90" t="s">
+        <v>104</v>
+      </c>
+      <c r="D90" s="2" t="s">
+        <v>797</v>
+      </c>
+      <c r="E90" s="3">
+        <v>15</v>
+      </c>
+      <c r="F90" s="4">
+        <v>9.11</v>
+      </c>
+      <c r="G90" s="3"/>
+      <c r="H90" s="3"/>
+      <c r="I90" s="3">
+        <v>2.52</v>
+      </c>
+      <c r="J90" s="3">
+        <v>0.96</v>
+      </c>
+      <c r="K90" s="3"/>
+      <c r="L90" s="3"/>
+      <c r="M90" s="3"/>
+      <c r="N90" s="3"/>
+      <c r="O90" s="2" t="s">
+        <v>798</v>
+      </c>
+    </row>
+    <row r="91" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A91" t="s">
+        <v>992</v>
+      </c>
+      <c r="B91" t="s">
+        <v>989</v>
+      </c>
+      <c r="C91" t="s">
+        <v>51</v>
+      </c>
+      <c r="D91" s="2" t="s">
+        <v>825</v>
+      </c>
+      <c r="E91" s="3">
+        <v>15.56</v>
+      </c>
+      <c r="F91" s="4">
+        <v>163.33</v>
+      </c>
+      <c r="G91" s="3"/>
+      <c r="H91" s="3"/>
+      <c r="I91" s="3">
+        <v>0</v>
+      </c>
+      <c r="J91" s="3">
+        <v>0</v>
+      </c>
+      <c r="K91" s="3"/>
+      <c r="L91" s="3"/>
+      <c r="M91" s="3"/>
+      <c r="N91" s="3"/>
+      <c r="O91" s="2" t="s">
+        <v>826</v>
+      </c>
+    </row>
+    <row r="92" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A92" t="s">
+        <v>990</v>
+      </c>
+      <c r="B92" t="s">
+        <v>991</v>
+      </c>
+      <c r="C92" t="s">
+        <v>46</v>
+      </c>
+      <c r="D92" s="2" t="s">
+        <v>829</v>
+      </c>
+      <c r="E92" s="3">
+        <v>15.7</v>
+      </c>
+      <c r="F92" s="4">
+        <v>8.48</v>
+      </c>
+      <c r="G92" s="3"/>
+      <c r="H92" s="3"/>
+      <c r="I92" s="3">
+        <v>-0.6</v>
+      </c>
+      <c r="J92" s="3">
+        <v>-2.51</v>
+      </c>
+      <c r="K92" s="3"/>
+      <c r="L92" s="3"/>
+      <c r="M92" s="3"/>
+      <c r="N92" s="3"/>
+      <c r="O92" s="2" t="s">
+        <v>830</v>
+      </c>
+    </row>
+    <row r="93" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A93" t="s">
+        <v>990</v>
+      </c>
+      <c r="B93" t="s">
+        <v>991</v>
+      </c>
+      <c r="C93" t="s">
+        <v>46</v>
+      </c>
+      <c r="D93" s="2" t="s">
+        <v>833</v>
+      </c>
+      <c r="E93" s="3">
+        <v>15.75</v>
+      </c>
+      <c r="F93" s="4">
+        <v>25.72</v>
+      </c>
+      <c r="G93" s="3"/>
+      <c r="H93" s="3"/>
+      <c r="I93" s="3">
+        <v>5.9</v>
+      </c>
+      <c r="J93" s="3">
+        <v>2.7</v>
+      </c>
+      <c r="K93" s="3"/>
+      <c r="L93" s="3"/>
+      <c r="M93" s="3"/>
+      <c r="N93" s="3"/>
+      <c r="O93" s="2" t="s">
+        <v>834</v>
+      </c>
+    </row>
+    <row r="94" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A94" t="s">
+        <v>404</v>
+      </c>
+      <c r="B94" t="s">
+        <v>989</v>
+      </c>
+      <c r="C94" t="s">
+        <v>404</v>
+      </c>
+      <c r="D94" s="2" t="s">
+        <v>840</v>
+      </c>
+      <c r="E94" s="3">
+        <v>15.98</v>
+      </c>
+      <c r="F94" s="4">
+        <v>216.94</v>
+      </c>
+      <c r="G94" s="3"/>
+      <c r="H94" s="3"/>
+      <c r="I94" s="3">
+        <v>1.18</v>
+      </c>
+      <c r="J94" s="3">
+        <v>0.9</v>
+      </c>
+      <c r="K94" s="3"/>
+      <c r="L94" s="3"/>
+      <c r="M94" s="3"/>
+      <c r="N94" s="3"/>
+      <c r="O94" s="2" t="s">
+        <v>841</v>
+      </c>
+    </row>
+    <row r="95" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A95" t="s">
+        <v>992</v>
+      </c>
+      <c r="B95" t="s">
+        <v>989</v>
+      </c>
+      <c r="C95" t="s">
+        <v>51</v>
+      </c>
+      <c r="D95" s="2" t="s">
+        <v>842</v>
+      </c>
+      <c r="E95" s="3">
+        <v>16.03</v>
+      </c>
+      <c r="F95" s="4">
+        <v>134.57</v>
+      </c>
+      <c r="G95" s="3"/>
+      <c r="H95" s="3"/>
+      <c r="I95" s="3">
+        <v>0.36</v>
+      </c>
+      <c r="J95" s="3">
+        <v>0.44</v>
+      </c>
+      <c r="K95" s="3"/>
+      <c r="L95" s="3"/>
+      <c r="M95" s="3"/>
+      <c r="N95" s="3"/>
+      <c r="O95" s="2" t="s">
+        <v>843</v>
+      </c>
+    </row>
+    <row r="96" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A96" t="s">
+        <v>990</v>
+      </c>
+      <c r="B96" t="s">
+        <v>993</v>
+      </c>
+      <c r="C96" t="s">
+        <v>72</v>
+      </c>
+      <c r="D96" s="2" t="s">
+        <v>850</v>
+      </c>
+      <c r="E96" s="3">
+        <v>16.18</v>
+      </c>
+      <c r="F96" s="4">
+        <v>16.11</v>
+      </c>
+      <c r="G96" s="3"/>
+      <c r="H96" s="3"/>
+      <c r="I96" s="3">
+        <v>6.92</v>
+      </c>
+      <c r="J96" s="3">
+        <v>4.35</v>
+      </c>
+      <c r="K96" s="3"/>
+      <c r="L96" s="3"/>
+      <c r="M96" s="3"/>
+      <c r="N96" s="3"/>
+      <c r="O96" s="2" t="s">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="97" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A97" t="s">
+        <v>404</v>
+      </c>
+      <c r="B97" t="s">
+        <v>989</v>
+      </c>
+      <c r="C97" t="s">
+        <v>404</v>
+      </c>
+      <c r="D97" s="2" t="s">
+        <v>852</v>
+      </c>
+      <c r="E97" s="3">
+        <v>16.19</v>
+      </c>
+      <c r="F97" s="4">
+        <v>160.2</v>
+      </c>
+      <c r="G97" s="3"/>
+      <c r="H97" s="3"/>
+      <c r="I97" s="3">
+        <v>0</v>
+      </c>
+      <c r="J97" s="3">
+        <v>0</v>
+      </c>
+      <c r="K97" s="3"/>
+      <c r="L97" s="3"/>
+      <c r="M97" s="3"/>
+      <c r="N97" s="3"/>
+      <c r="O97" s="2" t="s">
+        <v>853</v>
+      </c>
+    </row>
+    <row r="98" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A98" t="s">
+        <v>990</v>
+      </c>
+      <c r="B98" t="s">
+        <v>991</v>
+      </c>
+      <c r="C98" t="s">
+        <v>190</v>
+      </c>
+      <c r="D98" s="2" t="s">
+        <v>860</v>
+      </c>
+      <c r="E98" s="3">
+        <v>16.64</v>
+      </c>
+      <c r="F98" s="4">
+        <v>1326</v>
+      </c>
+      <c r="G98" s="3"/>
+      <c r="H98" s="3"/>
+      <c r="I98" s="3">
+        <v>11.05</v>
+      </c>
+      <c r="J98" s="3">
+        <v>10.23</v>
+      </c>
+      <c r="K98" s="3"/>
+      <c r="L98" s="3"/>
+      <c r="M98" s="3"/>
+      <c r="N98" s="3"/>
+      <c r="O98" s="2" t="s">
+        <v>861</v>
+      </c>
+    </row>
+    <row r="99" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A99" t="s">
+        <v>104</v>
+      </c>
+      <c r="B99" t="s">
+        <v>989</v>
+      </c>
+      <c r="C99" t="s">
+        <v>104</v>
+      </c>
+      <c r="D99" s="2" t="s">
+        <v>866</v>
+      </c>
+      <c r="E99" s="3">
+        <v>17</v>
+      </c>
+      <c r="F99" s="4">
+        <v>25.79</v>
+      </c>
+      <c r="G99" s="3"/>
+      <c r="H99" s="3"/>
+      <c r="I99" s="3">
+        <v>15.92</v>
+      </c>
+      <c r="J99" s="3">
+        <v>12.91</v>
+      </c>
+      <c r="K99" s="3"/>
+      <c r="L99" s="3"/>
+      <c r="M99" s="3"/>
+      <c r="N99" s="3"/>
+      <c r="O99" s="2" t="s">
+        <v>867</v>
+      </c>
+    </row>
+    <row r="100" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A100" t="s">
+        <v>992</v>
+      </c>
+      <c r="B100" t="s">
+        <v>989</v>
+      </c>
+      <c r="C100" t="s">
+        <v>158</v>
+      </c>
+      <c r="D100" s="2" t="s">
+        <v>868</v>
+      </c>
+      <c r="E100" s="3">
+        <v>17</v>
+      </c>
+      <c r="F100" s="4">
+        <v>20532.6</v>
+      </c>
+      <c r="G100" s="3"/>
+      <c r="H100" s="3"/>
+      <c r="I100" s="3">
+        <v>7.27</v>
+      </c>
+      <c r="J100" s="3">
+        <v>6.5</v>
+      </c>
+      <c r="K100" s="3"/>
+      <c r="L100" s="3"/>
+      <c r="M100" s="3"/>
+      <c r="N100" s="3"/>
+      <c r="O100" s="2" t="s">
+        <v>869</v>
+      </c>
+    </row>
+    <row r="101" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A101" t="s">
+        <v>24</v>
+      </c>
+      <c r="B101" t="s">
+        <v>989</v>
+      </c>
+      <c r="C101" t="s">
+        <v>24</v>
+      </c>
+      <c r="D101" s="2" t="s">
+        <v>878</v>
+      </c>
+      <c r="E101" s="3">
+        <v>17.13</v>
+      </c>
+      <c r="F101" s="4">
+        <v>38.01</v>
+      </c>
+      <c r="G101" s="3"/>
+      <c r="H101" s="3"/>
+      <c r="I101" s="3">
+        <v>9.37</v>
+      </c>
+      <c r="J101" s="3">
+        <v>6.05</v>
+      </c>
+      <c r="K101" s="3"/>
+      <c r="L101" s="3"/>
+      <c r="M101" s="3"/>
+      <c r="N101" s="3"/>
+      <c r="O101" s="2" t="s">
+        <v>879</v>
+      </c>
+    </row>
+    <row r="102" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A102" t="s">
+        <v>104</v>
+      </c>
+      <c r="B102" t="s">
+        <v>989</v>
+      </c>
+      <c r="C102" t="s">
+        <v>104</v>
+      </c>
+      <c r="D102" s="2" t="s">
+        <v>886</v>
+      </c>
+      <c r="E102" s="3">
+        <v>17.25</v>
+      </c>
+      <c r="F102" s="4">
+        <v>23.45</v>
+      </c>
+      <c r="G102" s="3"/>
+      <c r="H102" s="3"/>
+      <c r="I102" s="3">
+        <v>5.16</v>
+      </c>
+      <c r="J102" s="3">
+        <v>3.35</v>
+      </c>
+      <c r="K102" s="3"/>
+      <c r="L102" s="3"/>
+      <c r="M102" s="3"/>
+      <c r="N102" s="3"/>
+      <c r="O102" s="2" t="s">
+        <v>887</v>
+      </c>
+    </row>
+    <row r="103" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A103" t="s">
+        <v>992</v>
+      </c>
+      <c r="B103" t="s">
+        <v>989</v>
+      </c>
+      <c r="C103" t="s">
+        <v>51</v>
+      </c>
+      <c r="D103" s="2" t="s">
+        <v>903</v>
+      </c>
+      <c r="E103" s="3">
+        <v>17.7</v>
+      </c>
+      <c r="F103" s="4">
+        <v>67.45</v>
+      </c>
+      <c r="G103" s="3"/>
+      <c r="H103" s="3"/>
+      <c r="I103" s="3">
+        <v>8.2</v>
+      </c>
+      <c r="J103" s="3">
+        <v>6.75</v>
+      </c>
+      <c r="K103" s="3"/>
+      <c r="L103" s="3"/>
+      <c r="M103" s="3"/>
+      <c r="N103" s="3"/>
+      <c r="O103" s="2" t="s">
+        <v>904</v>
+      </c>
+    </row>
+    <row r="104" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A104" t="s">
+        <v>992</v>
+      </c>
+      <c r="B104" t="s">
+        <v>989</v>
+      </c>
+      <c r="C104" t="s">
+        <v>158</v>
+      </c>
+      <c r="D104" s="2" t="s">
+        <v>919</v>
+      </c>
+      <c r="E104" s="3">
+        <v>17.94</v>
+      </c>
+      <c r="F104" s="4">
+        <v>485.51</v>
+      </c>
+      <c r="G104" s="3"/>
+      <c r="H104" s="3"/>
+      <c r="I104" s="3">
+        <v>6.06</v>
+      </c>
+      <c r="J104" s="3">
+        <v>4.4</v>
+      </c>
+      <c r="K104" s="3"/>
+      <c r="L104" s="3"/>
+      <c r="M104" s="3"/>
+      <c r="N104" s="3"/>
+      <c r="O104" s="2" t="s">
+        <v>920</v>
+      </c>
+    </row>
+    <row r="105" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A105" t="s">
+        <v>990</v>
+      </c>
+      <c r="B105" t="s">
+        <v>997</v>
+      </c>
+      <c r="C105" t="s">
+        <v>220</v>
+      </c>
+      <c r="D105" s="2" t="s">
+        <v>929</v>
+      </c>
+      <c r="E105" s="3">
+        <v>18.18</v>
+      </c>
+      <c r="F105" s="4">
+        <v>199.98</v>
+      </c>
+      <c r="G105" s="3"/>
+      <c r="H105" s="3"/>
+      <c r="I105" s="3">
+        <v>18.06</v>
+      </c>
+      <c r="J105" s="3">
+        <v>13.23</v>
+      </c>
+      <c r="K105" s="3"/>
+      <c r="L105" s="3"/>
+      <c r="M105" s="3"/>
+      <c r="N105" s="3"/>
+      <c r="O105" s="2" t="s">
+        <v>930</v>
+      </c>
+    </row>
+    <row r="106" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A106" t="s">
+        <v>990</v>
+      </c>
+      <c r="B106" t="s">
+        <v>991</v>
+      </c>
+      <c r="C106" t="s">
+        <v>190</v>
+      </c>
+      <c r="D106" s="2" t="s">
+        <v>933</v>
+      </c>
+      <c r="E106" s="3">
+        <v>18.23</v>
+      </c>
+      <c r="F106" s="4">
+        <v>182.93</v>
+      </c>
+      <c r="G106" s="3"/>
+      <c r="H106" s="3"/>
+      <c r="I106" s="3">
+        <v>12.82</v>
+      </c>
+      <c r="J106" s="3">
+        <v>10.23</v>
+      </c>
+      <c r="K106" s="3"/>
+      <c r="L106" s="3"/>
+      <c r="M106" s="3"/>
+      <c r="N106" s="3"/>
+      <c r="O106" s="2" t="s">
+        <v>934</v>
+      </c>
+    </row>
+    <row r="107" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A107" t="s">
+        <v>998</v>
+      </c>
+      <c r="B107" t="s">
+        <v>989</v>
+      </c>
+      <c r="C107" t="s">
+        <v>939</v>
+      </c>
+      <c r="D107" s="2" t="s">
+        <v>940</v>
+      </c>
+      <c r="E107" s="3">
+        <v>18.3</v>
+      </c>
+      <c r="F107" s="4">
+        <v>44.79</v>
+      </c>
+      <c r="G107" s="3"/>
+      <c r="H107" s="3"/>
+      <c r="I107" s="3">
+        <v>5.08</v>
+      </c>
+      <c r="J107" s="3">
+        <v>1.51</v>
+      </c>
+      <c r="K107" s="3"/>
+      <c r="L107" s="3"/>
+      <c r="M107" s="3"/>
+      <c r="N107" s="3"/>
+      <c r="O107" s="2" t="s">
+        <v>941</v>
+      </c>
+    </row>
+    <row r="108" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A108" t="s">
+        <v>992</v>
+      </c>
+      <c r="B108" t="s">
+        <v>989</v>
+      </c>
+      <c r="C108" t="s">
+        <v>51</v>
+      </c>
+      <c r="D108" s="2" t="s">
+        <v>944</v>
+      </c>
+      <c r="E108" s="3">
+        <v>18.39</v>
+      </c>
+      <c r="F108" s="4">
+        <v>101.8</v>
+      </c>
+      <c r="G108" s="3"/>
+      <c r="H108" s="3"/>
+      <c r="I108" s="3">
+        <v>3.15</v>
+      </c>
+      <c r="J108" s="3">
+        <v>0.98</v>
+      </c>
+      <c r="K108" s="3"/>
+      <c r="L108" s="3"/>
+      <c r="M108" s="3"/>
+      <c r="N108" s="3"/>
+      <c r="O108" s="2" t="s">
+        <v>945</v>
+      </c>
+    </row>
+    <row r="109" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A109" t="s">
+        <v>990</v>
+      </c>
+      <c r="B109" t="s">
+        <v>991</v>
+      </c>
+      <c r="C109" t="s">
+        <v>46</v>
+      </c>
+      <c r="D109" s="2" t="s">
+        <v>954</v>
+      </c>
+      <c r="E109" s="3">
+        <v>18.5</v>
+      </c>
+      <c r="F109" s="4">
+        <v>24.12</v>
+      </c>
+      <c r="G109" s="3"/>
+      <c r="H109" s="3"/>
+      <c r="I109" s="3">
+        <v>3.51</v>
+      </c>
+      <c r="J109" s="3">
+        <v>2.23</v>
+      </c>
+      <c r="K109" s="3"/>
+      <c r="L109" s="3"/>
+      <c r="M109" s="3"/>
+      <c r="N109" s="3"/>
+      <c r="O109" s="2" t="s">
+        <v>955</v>
+      </c>
+    </row>
+    <row r="110" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A110" t="s">
+        <v>24</v>
+      </c>
+      <c r="B110" t="s">
+        <v>989</v>
+      </c>
+      <c r="C110" t="s">
+        <v>24</v>
+      </c>
+      <c r="D110" s="2" t="s">
+        <v>960</v>
+      </c>
+      <c r="E110" s="3">
+        <v>18.71</v>
+      </c>
+      <c r="F110" s="4">
+        <v>44.36</v>
+      </c>
+      <c r="G110" s="3"/>
+      <c r="H110" s="3"/>
+      <c r="I110" s="3">
+        <v>20.08</v>
+      </c>
+      <c r="J110" s="3">
+        <v>17.63</v>
+      </c>
+      <c r="K110" s="3"/>
+      <c r="L110" s="3"/>
+      <c r="M110" s="3"/>
+      <c r="N110" s="3"/>
+      <c r="O110" s="2" t="s">
+        <v>961</v>
+      </c>
+    </row>
+    <row r="111" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A111" t="s">
+        <v>998</v>
+      </c>
+      <c r="B111" t="s">
+        <v>989</v>
+      </c>
+      <c r="C111" t="s">
+        <v>939</v>
+      </c>
+      <c r="D111" s="2" t="s">
+        <v>964</v>
+      </c>
+      <c r="E111" s="3">
+        <v>19</v>
+      </c>
+      <c r="F111" s="4">
+        <v>10.95</v>
+      </c>
+      <c r="G111" s="3"/>
+      <c r="H111" s="3"/>
+      <c r="I111" s="3">
+        <v>0.89</v>
+      </c>
+      <c r="J111" s="3">
+        <v>0.84</v>
+      </c>
+      <c r="K111" s="3"/>
+      <c r="L111" s="3"/>
+      <c r="M111" s="3"/>
+      <c r="N111" s="3"/>
+      <c r="O111" s="2" t="s">
+        <v>965</v>
+      </c>
+    </row>
+    <row r="112" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A112" t="s">
+        <v>990</v>
+      </c>
+      <c r="B112" t="s">
+        <v>991</v>
+      </c>
+      <c r="C112" t="s">
+        <v>190</v>
+      </c>
+      <c r="D112" s="2" t="s">
+        <v>966</v>
+      </c>
+      <c r="E112" s="3">
+        <v>19</v>
+      </c>
+      <c r="F112" s="4">
+        <v>44.14</v>
+      </c>
+      <c r="G112" s="3"/>
+      <c r="H112" s="3"/>
+      <c r="I112" s="3">
+        <v>0</v>
+      </c>
+      <c r="J112" s="3">
+        <v>0</v>
+      </c>
+      <c r="K112" s="3"/>
+      <c r="L112" s="3"/>
+      <c r="M112" s="3"/>
+      <c r="N112" s="3"/>
+      <c r="O112" s="2" t="s">
+        <v>967</v>
+      </c>
+    </row>
+    <row r="113" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A113" t="s">
+        <v>994</v>
+      </c>
+      <c r="B113" t="s">
+        <v>989</v>
+      </c>
+      <c r="C113" t="s">
+        <v>968</v>
+      </c>
+      <c r="D113" s="2" t="s">
+        <v>969</v>
+      </c>
+      <c r="E113" s="3">
+        <v>19.19</v>
+      </c>
+      <c r="F113" s="4">
+        <v>4587.69</v>
+      </c>
+      <c r="G113" s="3"/>
+      <c r="H113" s="3"/>
+      <c r="I113" s="3">
+        <v>2.15</v>
+      </c>
+      <c r="J113" s="3">
+        <v>4.64</v>
+      </c>
+      <c r="K113" s="3"/>
+      <c r="L113" s="3"/>
+      <c r="M113" s="3"/>
+      <c r="N113" s="3"/>
+      <c r="O113" s="2" t="s">
+        <v>970</v>
+      </c>
+    </row>
+    <row r="114" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A114" t="s">
+        <v>404</v>
+      </c>
+      <c r="B114" t="s">
+        <v>989</v>
+      </c>
+      <c r="C114" t="s">
+        <v>404</v>
+      </c>
+      <c r="D114" s="2" t="s">
+        <v>975</v>
+      </c>
+      <c r="E114" s="3">
+        <v>19.41</v>
+      </c>
+      <c r="F114" s="4">
+        <v>8027.53</v>
+      </c>
+      <c r="G114" s="3"/>
+      <c r="H114" s="3"/>
+      <c r="I114" s="3">
+        <v>0.46</v>
+      </c>
+      <c r="J114" s="3">
+        <v>0.13</v>
+      </c>
+      <c r="K114" s="3"/>
+      <c r="L114" s="3"/>
+      <c r="M114" s="3"/>
+      <c r="N114" s="3"/>
+      <c r="O114" s="2" t="s">
+        <v>976</v>
+      </c>
+    </row>
+    <row r="115" ht="32" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A115" s="5" t="s">
+        <v>999</v>
+      </c>
+      <c r="B115" s="5"/>
+      <c r="C115" s="5"/>
+      <c r="D115" s="5"/>
+      <c r="E115" s="5"/>
+      <c r="F115" s="5"/>
+      <c r="G115" s="5"/>
+      <c r="H115" s="5"/>
+      <c r="I115" s="5"/>
+      <c r="J115" s="5"/>
+      <c r="K115" s="5"/>
+      <c r="L115" s="5"/>
+      <c r="M115" s="5"/>
+      <c r="N115" s="5"/>
+      <c r="O115" s="5"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:O1"/>
+  <mergeCells count="1">
+    <mergeCell ref="A115:O115"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="D2" r:id="rId1" tooltip="https://www.indmoney.com/stocks/welcure-drugs-and-pharmaceuticals-ltd-share-price"/>
+    <hyperlink ref="O2" r:id="rId2" tooltip="https://www.indmoney.com/stocks/welcure-drugs-and-pharmaceuticals-ltd-share-price"/>
+    <hyperlink ref="D3" r:id="rId3" tooltip="https://www.indmoney.com/stocks/remedium-lifecare-ltd-share-price"/>
+    <hyperlink ref="O3" r:id="rId4" tooltip="https://www.indmoney.com/stocks/remedium-lifecare-ltd-share-price"/>
+    <hyperlink ref="D4" r:id="rId5" tooltip="https://www.indmoney.com/stocks/rajnish-wellness-ltd-share-price"/>
+    <hyperlink ref="O4" r:id="rId6" tooltip="https://www.indmoney.com/stocks/rajnish-wellness-ltd-share-price"/>
+    <hyperlink ref="D5" r:id="rId7" tooltip="https://www.indmoney.com/stocks/western-ministil-ltd-share-price"/>
+    <hyperlink ref="O5" r:id="rId8" tooltip="https://www.indmoney.com/stocks/western-ministil-ltd-share-price"/>
+    <hyperlink ref="D6" r:id="rId9" tooltip="https://www.indmoney.com/stocks/unison-metals-ltd-share-price"/>
+    <hyperlink ref="O6" r:id="rId10" tooltip="https://www.indmoney.com/stocks/unison-metals-ltd-share-price"/>
+    <hyperlink ref="D7" r:id="rId11" tooltip="https://www.indmoney.com/stocks/navkar-urbanstructure-ltd-share-price"/>
+    <hyperlink ref="O7" r:id="rId12" tooltip="https://www.indmoney.com/stocks/navkar-urbanstructure-ltd-share-price"/>
+    <hyperlink ref="D8" r:id="rId13" tooltip="https://www.indmoney.com/stocks/sprayking-ltd-share-price"/>
+    <hyperlink ref="O8" r:id="rId14" tooltip="https://www.indmoney.com/stocks/sprayking-ltd-share-price"/>
+    <hyperlink ref="D9" r:id="rId15" tooltip="https://www.indmoney.com/stocks/ducon-infratechnologies-ltd-share-price"/>
+    <hyperlink ref="O9" r:id="rId16" tooltip="https://www.indmoney.com/stocks/ducon-infratechnologies-ltd-share-price"/>
+    <hyperlink ref="D10" r:id="rId17" tooltip="https://www.indmoney.com/stocks/family-care-hospitals-ltd-share-price"/>
+    <hyperlink ref="O10" r:id="rId18" tooltip="https://www.indmoney.com/stocks/family-care-hospitals-ltd-share-price"/>
+    <hyperlink ref="D11" r:id="rId19" tooltip="https://www.indmoney.com/stocks/ilandfs-transportation-networks-ltd-share-price"/>
+    <hyperlink ref="O11" r:id="rId20" tooltip="https://www.indmoney.com/stocks/ilandfs-transportation-networks-ltd-share-price"/>
+    <hyperlink ref="D12" r:id="rId21" tooltip="https://www.indmoney.com/stocks/ankit-metal-and-power-ltd-share-price"/>
+    <hyperlink ref="O12" r:id="rId22" tooltip="https://www.indmoney.com/stocks/ankit-metal-and-power-ltd-share-price"/>
+    <hyperlink ref="D13" r:id="rId23" tooltip="https://www.indmoney.com/stocks/parsvnath-developers-ltd-share-price"/>
+    <hyperlink ref="O13" r:id="rId24" tooltip="https://www.indmoney.com/stocks/parsvnath-developers-ltd-share-price"/>
+    <hyperlink ref="D14" r:id="rId25" tooltip="https://www.indmoney.com/stocks/davangere-sugar-company-ltd-share-price"/>
+    <hyperlink ref="O14" r:id="rId26" tooltip="https://www.indmoney.com/stocks/davangere-sugar-company-ltd-share-price"/>
+    <hyperlink ref="D15" r:id="rId27" tooltip="https://www.indmoney.com/stocks/transgene-biotek-ltd-share-price"/>
+    <hyperlink ref="O15" r:id="rId28" tooltip="https://www.indmoney.com/stocks/transgene-biotek-ltd-share-price"/>
+    <hyperlink ref="D16" r:id="rId29" tooltip="https://www.indmoney.com/stocks/gvk-power-and-infrastructure-ltd-share-price"/>
+    <hyperlink ref="O16" r:id="rId30" tooltip="https://www.indmoney.com/stocks/gvk-power-and-infrastructure-ltd-share-price"/>
+    <hyperlink ref="D17" r:id="rId31" tooltip="https://www.indmoney.com/stocks/sadbhav-infrastructure-projects-ltd-share-price"/>
+    <hyperlink ref="O17" r:id="rId32" tooltip="https://www.indmoney.com/stocks/sadbhav-infrastructure-projects-ltd-share-price"/>
+    <hyperlink ref="D18" r:id="rId33" tooltip="https://www.indmoney.com/stocks/alliance-integrated-metaliks-ltd-share-price"/>
+    <hyperlink ref="O18" r:id="rId34" tooltip="https://www.indmoney.com/stocks/alliance-integrated-metaliks-ltd-share-price"/>
+    <hyperlink ref="D19" r:id="rId35" tooltip="https://www.indmoney.com/stocks/shah-metacorp-ltd-share-price"/>
+    <hyperlink ref="O19" r:id="rId36" tooltip="https://www.indmoney.com/stocks/shah-metacorp-ltd-share-price"/>
+    <hyperlink ref="D20" r:id="rId37" tooltip="https://www.indmoney.com/stocks/facor-alloys-ltd-share-price"/>
+    <hyperlink ref="O20" r:id="rId38" tooltip="https://www.indmoney.com/stocks/facor-alloys-ltd-share-price"/>
+    <hyperlink ref="D21" r:id="rId39" tooltip="https://www.indmoney.com/stocks/mishtann-foods-ltd-share-price"/>
+    <hyperlink ref="O21" r:id="rId40" tooltip="https://www.indmoney.com/stocks/mishtann-foods-ltd-share-price"/>
+    <hyperlink ref="D22" r:id="rId41" tooltip="https://www.indmoney.com/stocks/rajnandini-metal-ltd-share-price"/>
+    <hyperlink ref="O22" r:id="rId42" tooltip="https://www.indmoney.com/stocks/rajnandini-metal-ltd-share-price"/>
+    <hyperlink ref="D23" r:id="rId43" tooltip="https://www.indmoney.com/stocks/sarveshwar-foods-ltd-share-price"/>
+    <hyperlink ref="O23" r:id="rId44" tooltip="https://www.indmoney.com/stocks/sarveshwar-foods-ltd-share-price"/>
+    <hyperlink ref="D24" r:id="rId45" tooltip="https://www.indmoney.com/stocks/noida-toll-bridge-company-ltd-share-price"/>
+    <hyperlink ref="O24" r:id="rId46" tooltip="https://www.indmoney.com/stocks/noida-toll-bridge-company-ltd-share-price"/>
+    <hyperlink ref="D25" r:id="rId47" tooltip="https://www.indmoney.com/stocks/prakash-steelage-ltd-share-price"/>
+    <hyperlink ref="O25" r:id="rId48" tooltip="https://www.indmoney.com/stocks/prakash-steelage-ltd-share-price"/>
+    <hyperlink ref="D26" r:id="rId49" tooltip="https://www.indmoney.com/stocks/sacheta-metals-ltd-share-price"/>
+    <hyperlink ref="O26" r:id="rId50" tooltip="https://www.indmoney.com/stocks/sacheta-metals-ltd-share-price"/>
+    <hyperlink ref="D27" r:id="rId51" tooltip="https://www.indmoney.com/stocks/dhatre-udyog-ltd-share-price"/>
+    <hyperlink ref="O27" r:id="rId52" tooltip="https://www.indmoney.com/stocks/dhatre-udyog-ltd-share-price"/>
+    <hyperlink ref="D28" r:id="rId53" tooltip="https://www.indmoney.com/stocks/kamdhenu-ventures-ltd-share-price"/>
+    <hyperlink ref="O28" r:id="rId54" tooltip="https://www.indmoney.com/stocks/kamdhenu-ventures-ltd-share-price"/>
+    <hyperlink ref="D29" r:id="rId55" tooltip="https://www.indmoney.com/stocks/salasar-techno-engineering-ltd-share-price"/>
+    <hyperlink ref="O29" r:id="rId56" tooltip="https://www.indmoney.com/stocks/salasar-techno-engineering-ltd-share-price"/>
+    <hyperlink ref="D30" r:id="rId57" tooltip="https://www.indmoney.com/stocks/supreme-engineering-ltd-share-price"/>
+    <hyperlink ref="O30" r:id="rId58" tooltip="https://www.indmoney.com/stocks/supreme-engineering-ltd-share-price"/>
+    <hyperlink ref="D31" r:id="rId59" tooltip="https://www.indmoney.com/stocks/rama-steel-tubes-ltd-share-price"/>
+    <hyperlink ref="O31" r:id="rId60" tooltip="https://www.indmoney.com/stocks/rama-steel-tubes-ltd-share-price"/>
+    <hyperlink ref="D32" r:id="rId61" tooltip="https://www.indmoney.com/stocks/gian-lifecare-ltd-share-price"/>
+    <hyperlink ref="O32" r:id="rId62" tooltip="https://www.indmoney.com/stocks/gian-lifecare-ltd-share-price"/>
+    <hyperlink ref="D33" r:id="rId63" tooltip="https://www.indmoney.com/stocks/kritika-wires-ltd-share-price"/>
+    <hyperlink ref="O33" r:id="rId64" tooltip="https://www.indmoney.com/stocks/kritika-wires-ltd-share-price"/>
+    <hyperlink ref="D34" r:id="rId65" tooltip="https://www.indmoney.com/stocks/shyam-century-ferrous-ltd-share-price"/>
+    <hyperlink ref="O34" r:id="rId66" tooltip="https://www.indmoney.com/stocks/shyam-century-ferrous-ltd-share-price"/>
+    <hyperlink ref="D35" r:id="rId67" tooltip="https://www.indmoney.com/stocks/sepc-ltd-share-price"/>
+    <hyperlink ref="O35" r:id="rId68" tooltip="https://www.indmoney.com/stocks/sepc-ltd-share-price"/>
+    <hyperlink ref="D36" r:id="rId69" tooltip="https://www.indmoney.com/stocks/zenith-steel-pipes-and-industries-ltd-share-price"/>
+    <hyperlink ref="O36" r:id="rId70" tooltip="https://www.indmoney.com/stocks/zenith-steel-pipes-and-industries-ltd-share-price"/>
+    <hyperlink ref="D37" r:id="rId71" tooltip="https://www.indmoney.com/stocks/lasa-supergenerics-ltd-share-price"/>
+    <hyperlink ref="O37" r:id="rId72" tooltip="https://www.indmoney.com/stocks/lasa-supergenerics-ltd-share-price"/>
+    <hyperlink ref="D38" r:id="rId73" tooltip="https://www.indmoney.com/stocks/vivimed-labs-ltd-share-price"/>
+    <hyperlink ref="O38" r:id="rId74" tooltip="https://www.indmoney.com/stocks/vivimed-labs-ltd-share-price"/>
+    <hyperlink ref="D39" r:id="rId75" tooltip="https://www.indmoney.com/stocks/achyut-healthcare-ltd-share-price"/>
+    <hyperlink ref="O39" r:id="rId76" tooltip="https://www.indmoney.com/stocks/achyut-healthcare-ltd-share-price"/>
+    <hyperlink ref="D40" r:id="rId77" tooltip="https://www.indmoney.com/stocks/vista-pharmaceuticals-ltd-share-price"/>
+    <hyperlink ref="O40" r:id="rId78" tooltip="https://www.indmoney.com/stocks/vista-pharmaceuticals-ltd-share-price"/>
+    <hyperlink ref="D41" r:id="rId79" tooltip="https://www.indmoney.com/stocks/heera-ispat-ltd-share-price"/>
+    <hyperlink ref="O41" r:id="rId80" tooltip="https://www.indmoney.com/stocks/heera-ispat-ltd-share-price"/>
+    <hyperlink ref="D42" r:id="rId81" tooltip="https://www.indmoney.com/stocks/bothra-metals-and-alloys-ltd-share-price"/>
+    <hyperlink ref="O42" r:id="rId82" tooltip="https://www.indmoney.com/stocks/bothra-metals-and-alloys-ltd-share-price"/>
+    <hyperlink ref="D43" r:id="rId83" tooltip="https://www.indmoney.com/stocks/deepak-builders-and-engineers-india-ltd-share-price"/>
+    <hyperlink ref="O43" r:id="rId84" tooltip="https://www.indmoney.com/stocks/deepak-builders-and-engineers-india-ltd-share-price"/>
+    <hyperlink ref="D44" r:id="rId85" tooltip="https://www.indmoney.com/stocks/impex-ferro-tech-ltd-share-price"/>
+    <hyperlink ref="O44" r:id="rId86" tooltip="https://www.indmoney.com/stocks/impex-ferro-tech-ltd-share-price"/>
+    <hyperlink ref="D45" r:id="rId87" tooltip="https://www.indmoney.com/stocks/nila-infrastructures-ltd-share-price"/>
+    <hyperlink ref="O45" r:id="rId88" tooltip="https://www.indmoney.com/stocks/nila-infrastructures-ltd-share-price"/>
+    <hyperlink ref="D46" r:id="rId89" tooltip="https://www.indmoney.com/stocks/rattanindia-power-ltd-share-price"/>
+    <hyperlink ref="O46" r:id="rId90" tooltip="https://www.indmoney.com/stocks/rattanindia-power-ltd-share-price"/>
+    <hyperlink ref="D47" r:id="rId91" tooltip="https://www.indmoney.com/stocks/india-power-corporation-ltd-share-price"/>
+    <hyperlink ref="O47" r:id="rId92" tooltip="https://www.indmoney.com/stocks/india-power-corporation-ltd-share-price"/>
+    <hyperlink ref="D48" r:id="rId93" tooltip="https://www.indmoney.com/stocks/sadbhav-engineering-ltd-share-price"/>
+    <hyperlink ref="O48" r:id="rId94" tooltip="https://www.indmoney.com/stocks/sadbhav-engineering-ltd-share-price"/>
+    <hyperlink ref="D49" r:id="rId95" tooltip="https://www.indmoney.com/stocks/dr-lalchandani-labs-ltd-share-price"/>
+    <hyperlink ref="O49" r:id="rId96" tooltip="https://www.indmoney.com/stocks/dr-lalchandani-labs-ltd-share-price"/>
+    <hyperlink ref="D50" r:id="rId97" tooltip="https://www.indmoney.com/stocks/madhav-infra-projects-ltd-share-price"/>
+    <hyperlink ref="O50" r:id="rId98" tooltip="https://www.indmoney.com/stocks/madhav-infra-projects-ltd-share-price"/>
+    <hyperlink ref="D51" r:id="rId99" tooltip="https://www.indmoney.com/stocks/elitecon-international-ltd-share-price"/>
+    <hyperlink ref="O51" r:id="rId100" tooltip="https://www.indmoney.com/stocks/elitecon-international-ltd-share-price"/>
+    <hyperlink ref="D52" r:id="rId101" tooltip="https://www.indmoney.com/stocks/twamev-construction-and-infrastructure-ltd-share-price"/>
+    <hyperlink ref="O52" r:id="rId102" tooltip="https://www.indmoney.com/stocks/twamev-construction-and-infrastructure-ltd-share-price"/>
+    <hyperlink ref="D53" r:id="rId103" tooltip="https://www.indmoney.com/stocks/aditya-ispat-ltd-share-price"/>
+    <hyperlink ref="O53" r:id="rId104" tooltip="https://www.indmoney.com/stocks/aditya-ispat-ltd-share-price"/>
+    <hyperlink ref="D54" r:id="rId105" tooltip="https://www.indmoney.com/stocks/bharat-immunological-and-biological-corporation-ltd-share-price"/>
+    <hyperlink ref="O54" r:id="rId106" tooltip="https://www.indmoney.com/stocks/bharat-immunological-and-biological-corporation-ltd-share-price"/>
+    <hyperlink ref="D55" r:id="rId107" tooltip="https://www.indmoney.com/stocks/vaishali-pharma-ltd-share-price"/>
+    <hyperlink ref="O55" r:id="rId108" tooltip="https://www.indmoney.com/stocks/vaishali-pharma-ltd-share-price"/>
+    <hyperlink ref="D56" r:id="rId109" tooltip="https://www.indmoney.com/stocks/indowind-energy-ltd-share-price"/>
+    <hyperlink ref="O56" r:id="rId110" tooltip="https://www.indmoney.com/stocks/indowind-energy-ltd-share-price"/>
+    <hyperlink ref="D57" r:id="rId111" tooltip="https://www.indmoney.com/stocks/vallabh-steels-ltd-share-price"/>
+    <hyperlink ref="O57" r:id="rId112" tooltip="https://www.indmoney.com/stocks/vallabh-steels-ltd-share-price"/>
+    <hyperlink ref="D58" r:id="rId113" tooltip="https://www.indmoney.com/stocks/orient-green-power-company-ltd-share-price"/>
+    <hyperlink ref="O58" r:id="rId114" tooltip="https://www.indmoney.com/stocks/orient-green-power-company-ltd-share-price"/>
+    <hyperlink ref="D59" r:id="rId115" tooltip="https://www.indmoney.com/stocks/rajasthan-tube-manufacturing-co-ltd-share-price"/>
+    <hyperlink ref="O59" r:id="rId116" tooltip="https://www.indmoney.com/stocks/rajasthan-tube-manufacturing-co-ltd-share-price"/>
+    <hyperlink ref="D60" r:id="rId117" tooltip="https://www.indmoney.com/stocks/baroda-extrusion-ltd-share-price"/>
+    <hyperlink ref="O60" r:id="rId118" tooltip="https://www.indmoney.com/stocks/baroda-extrusion-ltd-share-price"/>
+    <hyperlink ref="D61" r:id="rId119" tooltip="https://www.indmoney.com/stocks/looks-health-services-ltd-share-price"/>
+    <hyperlink ref="O61" r:id="rId120" tooltip="https://www.indmoney.com/stocks/looks-health-services-ltd-share-price"/>
+    <hyperlink ref="D62" r:id="rId121" tooltip="https://www.indmoney.com/stocks/gennex-laboratories-ltd-share-price"/>
+    <hyperlink ref="O62" r:id="rId122" tooltip="https://www.indmoney.com/stocks/gennex-laboratories-ltd-share-price"/>
+    <hyperlink ref="D63" r:id="rId123" tooltip="https://www.indmoney.com/stocks/mahalaxmi-seamless-ltd-share-price"/>
+    <hyperlink ref="O63" r:id="rId124" tooltip="https://www.indmoney.com/stocks/mahalaxmi-seamless-ltd-share-price"/>
+    <hyperlink ref="D64" r:id="rId125" tooltip="https://www.indmoney.com/stocks/jfl-life-sciences-ltd-share-price"/>
+    <hyperlink ref="O64" r:id="rId126" tooltip="https://www.indmoney.com/stocks/jfl-life-sciences-ltd-share-price"/>
+    <hyperlink ref="D65" r:id="rId127" tooltip="https://www.indmoney.com/stocks/la-tim-metal-and-industries-ltd-share-price"/>
+    <hyperlink ref="O65" r:id="rId128" tooltip="https://www.indmoney.com/stocks/la-tim-metal-and-industries-ltd-share-price"/>
+    <hyperlink ref="D66" r:id="rId129" tooltip="https://www.indmoney.com/stocks/boston-commerce-limited-share-price"/>
+    <hyperlink ref="O66" r:id="rId130" tooltip="https://www.indmoney.com/stocks/boston-commerce-limited-share-price"/>
+    <hyperlink ref="D67" r:id="rId131" tooltip="https://www.indmoney.com/stocks/nectar-lifescience-ltd-share-price"/>
+    <hyperlink ref="O67" r:id="rId132" tooltip="https://www.indmoney.com/stocks/nectar-lifescience-ltd-share-price"/>
+    <hyperlink ref="D68" r:id="rId133" tooltip="https://www.indmoney.com/stocks/maruti-infrastructure-ltd-share-price"/>
+    <hyperlink ref="O68" r:id="rId134" tooltip="https://www.indmoney.com/stocks/maruti-infrastructure-ltd-share-price"/>
+    <hyperlink ref="D69" r:id="rId135" tooltip="https://www.indmoney.com/stocks/steel-exchange-india-ltd-share-price"/>
+    <hyperlink ref="O69" r:id="rId136" tooltip="https://www.indmoney.com/stocks/steel-exchange-india-ltd-share-price"/>
+    <hyperlink ref="D70" r:id="rId137" tooltip="https://www.indmoney.com/stocks/deccan-health-care-ltd-share-price"/>
+    <hyperlink ref="O70" r:id="rId138" tooltip="https://www.indmoney.com/stocks/deccan-health-care-ltd-share-price"/>
+    <hyperlink ref="D71" r:id="rId139" tooltip="https://www.indmoney.com/stocks/earthstahl-and-alloys-ltd-share-price"/>
+    <hyperlink ref="O71" r:id="rId140" tooltip="https://www.indmoney.com/stocks/earthstahl-and-alloys-ltd-share-price"/>
+    <hyperlink ref="D72" r:id="rId141" tooltip="https://www.indmoney.com/stocks/global-longlife-hospital-and-research-ltd-share-price"/>
+    <hyperlink ref="O72" r:id="rId142" tooltip="https://www.indmoney.com/stocks/global-longlife-hospital-and-research-ltd-share-price"/>
+    <hyperlink ref="D73" r:id="rId143" tooltip="https://www.indmoney.com/stocks/global-defence-industries-limited-share-price"/>
+    <hyperlink ref="O73" r:id="rId144" tooltip="https://www.indmoney.com/stocks/global-defence-industries-limited-share-price"/>
+    <hyperlink ref="D74" r:id="rId145" tooltip="https://www.indmoney.com/stocks/bihar-sponge-iron-ltd-share-price"/>
+    <hyperlink ref="O74" r:id="rId146" tooltip="https://www.indmoney.com/stocks/bihar-sponge-iron-ltd-share-price"/>
+    <hyperlink ref="D75" r:id="rId147" tooltip="https://www.indmoney.com/stocks/a-b-infrabuild-ltd-share-price"/>
+    <hyperlink ref="O75" r:id="rId148" tooltip="https://www.indmoney.com/stocks/a-b-infrabuild-ltd-share-price"/>
+    <hyperlink ref="D76" r:id="rId149" tooltip="https://www.indmoney.com/stocks/take-ltd-share-price"/>
+    <hyperlink ref="O76" r:id="rId150" tooltip="https://www.indmoney.com/stocks/take-ltd-share-price"/>
+    <hyperlink ref="D77" r:id="rId151" tooltip="https://www.indmoney.com/stocks/tejnaksh-healthcare-ltd-share-price"/>
+    <hyperlink ref="O77" r:id="rId152" tooltip="https://www.indmoney.com/stocks/tejnaksh-healthcare-ltd-share-price"/>
+    <hyperlink ref="D78" r:id="rId153" tooltip="https://www.indmoney.com/stocks/nova-iron-and-steel-ltd-share-price"/>
+    <hyperlink ref="O78" r:id="rId154" tooltip="https://www.indmoney.com/stocks/nova-iron-and-steel-ltd-share-price"/>
+    <hyperlink ref="D79" r:id="rId155" tooltip="https://www.indmoney.com/stocks/atal-realtech-ltd-share-price"/>
+    <hyperlink ref="O79" r:id="rId156" tooltip="https://www.indmoney.com/stocks/atal-realtech-ltd-share-price"/>
+    <hyperlink ref="D80" r:id="rId157" tooltip="https://www.indmoney.com/stocks/nidan-laboratories-and-healthcare-ltd-share-price"/>
+    <hyperlink ref="O80" r:id="rId158" tooltip="https://www.indmoney.com/stocks/nidan-laboratories-and-healthcare-ltd-share-price"/>
+    <hyperlink ref="D81" r:id="rId159" tooltip="https://www.indmoney.com/stocks/consolidated-construction-consortium-ltd-share-price"/>
+    <hyperlink ref="O81" r:id="rId160" tooltip="https://www.indmoney.com/stocks/consolidated-construction-consortium-ltd-share-price"/>
+    <hyperlink ref="D82" r:id="rId161" tooltip="https://www.indmoney.com/stocks/mukat-pipes-ltd-share-price"/>
+    <hyperlink ref="O82" r:id="rId162" tooltip="https://www.indmoney.com/stocks/mukat-pipes-ltd-share-price"/>
+    <hyperlink ref="D83" r:id="rId163" tooltip="https://www.indmoney.com/stocks/ind-renewable-energy-ltd-share-price"/>
+    <hyperlink ref="O83" r:id="rId164" tooltip="https://www.indmoney.com/stocks/ind-renewable-energy-ltd-share-price"/>
+    <hyperlink ref="D84" r:id="rId165" tooltip="https://www.indmoney.com/stocks/modern-steels-ltd-share-price"/>
+    <hyperlink ref="O84" r:id="rId166" tooltip="https://www.indmoney.com/stocks/modern-steels-ltd-share-price"/>
+    <hyperlink ref="D85" r:id="rId167" tooltip="https://www.indmoney.com/stocks/a2z-infra-engineering-ltd-share-price"/>
+    <hyperlink ref="O85" r:id="rId168" tooltip="https://www.indmoney.com/stocks/a2z-infra-engineering-ltd-share-price"/>
+    <hyperlink ref="D86" r:id="rId169" tooltip="https://www.indmoney.com/stocks/arcee-industries-ltd-share-price"/>
+    <hyperlink ref="O86" r:id="rId170" tooltip="https://www.indmoney.com/stocks/arcee-industries-ltd-share-price"/>
+    <hyperlink ref="D87" r:id="rId171" tooltip="https://www.indmoney.com/stocks/energy-development-company-ltd-share-price"/>
+    <hyperlink ref="O87" r:id="rId172" tooltip="https://www.indmoney.com/stocks/energy-development-company-ltd-share-price"/>
+    <hyperlink ref="D88" r:id="rId173" tooltip="https://www.indmoney.com/stocks/venmax-drugs-and-pharmaceuticals-ltd-share-price"/>
+    <hyperlink ref="O88" r:id="rId174" tooltip="https://www.indmoney.com/stocks/venmax-drugs-and-pharmaceuticals-ltd-share-price"/>
+    <hyperlink ref="D89" r:id="rId175" tooltip="https://www.indmoney.com/stocks/jaiprakash-power-ventures-ltd-share-price"/>
+    <hyperlink ref="O89" r:id="rId176" tooltip="https://www.indmoney.com/stocks/jaiprakash-power-ventures-ltd-share-price"/>
+    <hyperlink ref="D90" r:id="rId177" tooltip="https://www.indmoney.com/stocks/broach-lifecare-hospital-ltd-share-price"/>
+    <hyperlink ref="O90" r:id="rId178" tooltip="https://www.indmoney.com/stocks/broach-lifecare-hospital-ltd-share-price"/>
+    <hyperlink ref="D91" r:id="rId179" tooltip="https://www.indmoney.com/stocks/modulex-construction-technologies-ltd-share-price"/>
+    <hyperlink ref="O91" r:id="rId180" tooltip="https://www.indmoney.com/stocks/modulex-construction-technologies-ltd-share-price"/>
+    <hyperlink ref="D92" r:id="rId181" tooltip="https://www.indmoney.com/stocks/eastcoast-steel-ltd-share-price"/>
+    <hyperlink ref="O92" r:id="rId182" tooltip="https://www.indmoney.com/stocks/eastcoast-steel-ltd-share-price"/>
+    <hyperlink ref="D93" r:id="rId183" tooltip="https://www.indmoney.com/stocks/rathi-bars-ltd-share-price"/>
+    <hyperlink ref="O93" r:id="rId184" tooltip="https://www.indmoney.com/stocks/rathi-bars-ltd-share-price"/>
+    <hyperlink ref="D94" r:id="rId185" tooltip="https://www.indmoney.com/stocks/surana-telecom-and-power-ltd-share-price"/>
+    <hyperlink ref="O94" r:id="rId186" tooltip="https://www.indmoney.com/stocks/surana-telecom-and-power-ltd-share-price"/>
+    <hyperlink ref="D95" r:id="rId187" tooltip="https://www.indmoney.com/stocks/bharat-road-network-ltd-share-price"/>
+    <hyperlink ref="O95" r:id="rId188" tooltip="https://www.indmoney.com/stocks/bharat-road-network-ltd-share-price"/>
+    <hyperlink ref="D96" r:id="rId189" tooltip="https://www.indmoney.com/stocks/poojawestern-metaliks-ltd-share-price"/>
+    <hyperlink ref="O96" r:id="rId190" tooltip="https://www.indmoney.com/stocks/poojawestern-metaliks-ltd-share-price"/>
+    <hyperlink ref="D97" r:id="rId191" tooltip="https://www.indmoney.com/stocks/globus-power-generation-ltd-share-price"/>
+    <hyperlink ref="O97" r:id="rId192" tooltip="https://www.indmoney.com/stocks/globus-power-generation-ltd-share-price"/>
+    <hyperlink ref="D98" r:id="rId193" tooltip="https://www.indmoney.com/stocks/rhetan-tmt-ltd-share-price"/>
+    <hyperlink ref="O98" r:id="rId194" tooltip="https://www.indmoney.com/stocks/rhetan-tmt-ltd-share-price"/>
+    <hyperlink ref="D99" r:id="rId195" tooltip="https://www.indmoney.com/stocks/galaxy-medicare-ltd-share-price"/>
+    <hyperlink ref="O99" r:id="rId196" tooltip="https://www.indmoney.com/stocks/galaxy-medicare-ltd-share-price"/>
+    <hyperlink ref="D100" r:id="rId197" tooltip="https://www.indmoney.com/stocks/irb-infrastructure-developers-ltd-share-price"/>
+    <hyperlink ref="O100" r:id="rId198" tooltip="https://www.indmoney.com/stocks/irb-infrastructure-developers-ltd-share-price"/>
+    <hyperlink ref="D101" r:id="rId199" tooltip="https://www.indmoney.com/stocks/vivo-bio-tech-ltd-share-price"/>
+    <hyperlink ref="O101" r:id="rId200" tooltip="https://www.indmoney.com/stocks/vivo-bio-tech-ltd-share-price"/>
+    <hyperlink ref="D102" r:id="rId201" tooltip="https://www.indmoney.com/stocks/adeshwar-meditex-ltd-share-price"/>
+    <hyperlink ref="O102" r:id="rId202" tooltip="https://www.indmoney.com/stocks/adeshwar-meditex-ltd-share-price"/>
+    <hyperlink ref="D103" r:id="rId203" tooltip="https://www.indmoney.com/stocks/kandr-rail-engineering-ltd-share-price"/>
+    <hyperlink ref="O103" r:id="rId204" tooltip="https://www.indmoney.com/stocks/kandr-rail-engineering-ltd-share-price"/>
+    <hyperlink ref="D104" r:id="rId205" tooltip="https://www.indmoney.com/stocks/hazoor-multi-projects-ltd-share-price"/>
+    <hyperlink ref="O104" r:id="rId206" tooltip="https://www.indmoney.com/stocks/hazoor-multi-projects-ltd-share-price"/>
+    <hyperlink ref="D105" r:id="rId207" tooltip="https://www.indmoney.com/stocks/century-extrusions-ltd-share-price"/>
+    <hyperlink ref="O105" r:id="rId208" tooltip="https://www.indmoney.com/stocks/century-extrusions-ltd-share-price"/>
+    <hyperlink ref="D106" r:id="rId209" tooltip="https://www.indmoney.com/stocks/rudra-global-infra-products-ltd-share-price"/>
+    <hyperlink ref="O106" r:id="rId210" tooltip="https://www.indmoney.com/stocks/rudra-global-infra-products-ltd-share-price"/>
+    <hyperlink ref="D107" r:id="rId211" tooltip="https://www.indmoney.com/stocks/vms-industries-ltd-share-price"/>
+    <hyperlink ref="O107" r:id="rId212" tooltip="https://www.indmoney.com/stocks/vms-industries-ltd-share-price"/>
+    <hyperlink ref="D108" r:id="rId213" tooltip="https://www.indmoney.com/stocks/udayshivakumar-infra-ltd-share-price"/>
+    <hyperlink ref="O108" r:id="rId214" tooltip="https://www.indmoney.com/stocks/udayshivakumar-infra-ltd-share-price"/>
+    <hyperlink ref="D109" r:id="rId215" tooltip="https://www.indmoney.com/stocks/kalana-ispat-ltd-share-price"/>
+    <hyperlink ref="O109" r:id="rId216" tooltip="https://www.indmoney.com/stocks/kalana-ispat-ltd-share-price"/>
+    <hyperlink ref="D110" r:id="rId217" tooltip="https://www.indmoney.com/stocks/kabra-drugs-ltd-share-price"/>
+    <hyperlink ref="O110" r:id="rId218" tooltip="https://www.indmoney.com/stocks/kabra-drugs-ltd-share-price"/>
+    <hyperlink ref="D111" r:id="rId219" tooltip="https://www.indmoney.com/stocks/garware-marine-industries-ltd-share-price"/>
+    <hyperlink ref="O111" r:id="rId220" tooltip="https://www.indmoney.com/stocks/garware-marine-industries-ltd-share-price"/>
+    <hyperlink ref="D112" r:id="rId221" tooltip="https://www.indmoney.com/stocks/swastik-pipe-ltd-share-price"/>
+    <hyperlink ref="O112" r:id="rId222" tooltip="https://www.indmoney.com/stocks/swastik-pipe-ltd-share-price"/>
+    <hyperlink ref="D113" r:id="rId223" tooltip="https://www.indmoney.com/stocks/bajaj-hindusthan-sugar-ltd-share-price"/>
+    <hyperlink ref="O113" r:id="rId224" tooltip="https://www.indmoney.com/stocks/bajaj-hindusthan-sugar-ltd-share-price"/>
+    <hyperlink ref="D114" r:id="rId225" tooltip="https://www.indmoney.com/stocks/reliance-power-ltd-share-price"/>
+    <hyperlink ref="O114" r:id="rId226" tooltip="https://www.indmoney.com/stocks/reliance-power-ltd-share-price"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
 </file>
</xml_diff>